<commit_message>
front wheel hub assembly
</commit_message>
<xml_diff>
--- a/Shareef/Suspension Tools/3D_Suspension_Analyzer/3D_Suspension_Analyzer_V2.xlsx
+++ b/Shareef/Suspension Tools/3D_Suspension_Analyzer/3D_Suspension_Analyzer_V2.xlsx
@@ -8,15 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\share\OneDrive\Documents\Personal Projects\GOGO Kart\CAD\GOGO_KART_FSAE\Shareef\Suspension Tools\3D_Suspension_Analyzer\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7828737-E518-432B-B1CE-4C8080D7C9CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40DBD78C-914A-467D-903A-FC0135B077CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-135" yWindow="-135" windowWidth="38670" windowHeight="21150" xr2:uid="{9695B30A-B9BA-4C2C-80C9-40991A052BC6}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{9695B30A-B9BA-4C2C-80C9-40991A052BC6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1" sheetId="2" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -75,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="92">
   <si>
     <t>Value</t>
   </si>
@@ -348,6 +347,9 @@
   </si>
   <si>
     <t>Camber Angle</t>
+  </si>
+  <si>
+    <t>Camber-KPI Offset (deg)</t>
   </si>
 </sst>
 </file>
@@ -355,7 +357,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="175" formatCode="0.0"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -372,7 +374,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -409,8 +411,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -470,11 +478,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -487,6 +504,21 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -502,19 +534,13 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="175" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="175" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="175" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -655,7 +681,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'Sheet 1'!$H$4:$H$44</c:f>
+              <c:f>'Sheet 1'!$S$4:$S$44</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="41"/>
@@ -787,132 +813,132 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Sheet 1'!$I$4:$I$44</c:f>
+              <c:f>'Sheet 1'!$T$4:$T$44</c:f>
               <c:numCache>
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="41"/>
                 <c:pt idx="0">
-                  <c:v>5.0784445424152018</c:v>
+                  <c:v>-4.481455409386534</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.9929530523627381</c:v>
+                  <c:v>-4.5096282411695068</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4.9145587013259746</c:v>
+                  <c:v>-4.5337589113301595</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>4.8431988789515419</c:v>
+                  <c:v>-4.5539317551658343</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>4.7788169483417331</c:v>
+                  <c:v>-4.5702252042057925</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>4.7213623345594122</c:v>
+                  <c:v>-4.5827119694154002</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>4.6707906185819752</c:v>
+                  <c:v>-4.5914592125202569</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>4.6270636378975958</c:v>
+                  <c:v>-4.5965287054464969</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>4.5901495949651991</c:v>
+                  <c:v>-4.5979769778990534</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>4.5600231747982534</c:v>
+                  <c:v>-4.5958554531206639</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>4.5366656729775681</c:v>
+                  <c:v>-4.5902105718840218</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>4.5200651354569228</c:v>
+                  <c:v>-4.5810839047740481</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>4.5102165115946331</c:v>
+                  <c:v>-4.5685122528115603</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>4.5071218219256117</c:v>
+                  <c:v>-4.552527736461915</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>4.510790342286521</c:v>
+                  <c:v>-4.533157873055548</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>4.521238806021131</c:v>
+                  <c:v>-4.5104256426280429</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>4.5384916261219512</c:v>
+                  <c:v>-4.4843495421615902</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>4.562581139320443</c:v>
+                  <c:v>-4.4549436281809491</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>4.5935478743113354</c:v>
+                  <c:v>-4.4222175476229966</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>4.6314408465004711</c:v>
+                  <c:v>-4.3861765568610096</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>4.6763178818957858</c:v>
+                  <c:v>-4.346821528722181</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>4.7282459730292103</c:v>
+                  <c:v>-4.3041489472911785</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>4.787301670100236</c:v>
+                  <c:v>-4.258150890240632</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>4.8535715108811956</c:v>
+                  <c:v>-4.2088149983734144</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>4.9271524933254724</c:v>
+                  <c:v>-4.1561244320006185</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>5.0081525952775916</c:v>
+                  <c:v>-4.1000578137126542</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>5.096691346211756</c:v>
+                  <c:v>-4.0405891570269974</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>5.1929004565316337</c:v>
+                  <c:v>-3.9776877803165664</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>5.2969245106614267</c:v>
+                  <c:v>-3.9113182053348545</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>5.4089217309654174</c:v>
+                  <c:v>-3.8414400395590254</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>5.529064820462489</c:v>
+                  <c:v>-3.7680078414639691</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>5.6575418933853232</c:v>
+                  <c:v>-3.6909709677256304</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>5.7945575038849313</c:v>
+                  <c:v>-3.6102734012226483</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>5.9403337846479189</c:v>
+                  <c:v>-3.5258535585610882</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>6.0951117088974627</c:v>
+                  <c:v>-3.4376440756897959</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>6.2591524912573213</c:v>
+                  <c:v>-3.3455715699963791</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>6.4327391453079734</c:v>
+                  <c:v>-3.249556377075816</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>6.6161782184459792</c:v>
+                  <c:v>-3.1495122601440277</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>6.8098017279472227</c:v>
+                  <c:v>-3.0453460898189029</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>7.0139693260434051</c:v>
+                  <c:v>-2.9369574917140335</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>7.2290707264922318</c:v>
+                  <c:v>-2.8242384589742762</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1022,8 +1048,9 @@
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
           <a:noFill/>
-          <a:ln>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
             <a:noFill/>
+            <a:round/>
           </a:ln>
           <a:effectLst/>
         </c:spPr>
@@ -1092,7 +1119,15 @@
                 </a:pPr>
                 <a:r>
                   <a:rPr lang="en-US"/>
-                  <a:t>Kingpin Inclination (degrees)</a:t>
+                  <a:t>Camber</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" baseline="0"/>
+                  <a:t> </a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t> Angle (degrees)</a:t>
                 </a:r>
               </a:p>
               <a:p>
@@ -1815,7 +1850,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>6989576</xdr:colOff>
+      <xdr:colOff>6997196</xdr:colOff>
       <xdr:row>79</xdr:row>
       <xdr:rowOff>35960</xdr:rowOff>
     </xdr:to>
@@ -1858,10 +1893,10 @@
       <xdr:rowOff>100852</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>191569</xdr:colOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>102669</xdr:colOff>
       <xdr:row>71</xdr:row>
-      <xdr:rowOff>134694</xdr:rowOff>
+      <xdr:rowOff>140409</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1913,16 +1948,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>19</xdr:col>
-      <xdr:colOff>134469</xdr:colOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>817094</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>78440</xdr:rowOff>
+      <xdr:rowOff>189565</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>33</xdr:col>
-      <xdr:colOff>369793</xdr:colOff>
-      <xdr:row>34</xdr:row>
-      <xdr:rowOff>190499</xdr:rowOff>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2364,67 +2399,87 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{523DEDE4-CF63-4BE7-9597-216ED5BF300E}">
-  <dimension ref="C3:R46"/>
+  <dimension ref="C3:AC46"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="14.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="146" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="159" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13.42578125" customWidth="1"/>
-    <col min="8" max="9" width="15.7109375" customWidth="1"/>
+    <col min="8" max="8" width="15.7109375" customWidth="1"/>
+    <col min="9" max="9" width="10.7109375" customWidth="1"/>
     <col min="10" max="11" width="6.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.42578125" customWidth="1"/>
     <col min="13" max="13" width="8.140625" customWidth="1"/>
     <col min="14" max="14" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="27.7109375" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="38" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="35.42578125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="19" customWidth="1"/>
+    <col min="16" max="16" width="22.85546875" customWidth="1"/>
+    <col min="19" max="19" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="9.140625" customWidth="1"/>
+    <col min="22" max="22" width="9" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="32.28515625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="43.42578125" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="41.140625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="18.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="3:18" x14ac:dyDescent="0.25">
-      <c r="C3" s="6" t="s">
+    <row r="3" spans="3:29" x14ac:dyDescent="0.25">
+      <c r="C3" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="D3" s="6"/>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
-      <c r="H3" s="12" t="s">
+      <c r="D3" s="11"/>
+      <c r="E3" s="11"/>
+      <c r="F3" s="11"/>
+      <c r="H3" s="16" t="s">
+        <v>91</v>
+      </c>
+      <c r="I3" s="15"/>
+      <c r="J3" s="15"/>
+      <c r="K3" s="15"/>
+      <c r="L3" s="15"/>
+      <c r="M3" s="15"/>
+      <c r="N3" s="15"/>
+      <c r="O3" s="15"/>
+      <c r="P3" s="15"/>
+      <c r="S3" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="I3" s="12" t="s">
+      <c r="T3" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="J3" s="12" t="s">
+      <c r="U3" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="K3" s="12" t="s">
+      <c r="V3" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="L3" s="12" t="s">
+      <c r="W3" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="M3" s="12" t="s">
+      <c r="X3" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="N3" s="12" t="s">
+      <c r="Y3" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="O3" s="12" t="s">
+      <c r="Z3" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="P3" s="12" t="s">
+      <c r="AA3" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="Q3" s="12" t="s">
+      <c r="AB3" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="R3" s="12" t="s">
+      <c r="AC3" s="7" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="4" spans="3:18" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="4" spans="3:29" ht="15.75" x14ac:dyDescent="0.3">
       <c r="C4" s="2" t="s">
         <v>4</v>
       </c>
@@ -2437,51 +2492,62 @@
       <c r="F4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="H4" s="11">
+      <c r="H4" s="17">
+        <v>0</v>
+      </c>
+      <c r="I4" s="18"/>
+      <c r="J4" s="18"/>
+      <c r="K4" s="18"/>
+      <c r="L4" s="18"/>
+      <c r="M4" s="18"/>
+      <c r="N4" s="18"/>
+      <c r="O4" s="18"/>
+      <c r="P4" s="18"/>
+      <c r="S4" s="6">
         <v>20</v>
       </c>
-      <c r="I4" s="13">
-        <f>R4-5</f>
-        <v>5.0784445424152018</v>
-      </c>
-      <c r="J4" s="14">
-        <f>$D$5+$D$22*COS(RADIANS(H4))</f>
-        <v>242.82091344766073</v>
-      </c>
-      <c r="K4" s="14">
-        <f>$D$6+$D$22*SIN(RADIANS(H4))</f>
-        <v>151.98256132565808</v>
-      </c>
-      <c r="L4" s="14">
-        <f>SQRT((J4-$D$7)^2+(K4-$D$8)^2)</f>
-        <v>203.44629542829861</v>
-      </c>
-      <c r="M4" s="14">
-        <f>($D$23^2-$D$27^2+L4^2)/(2*L4)</f>
-        <v>173.24079304344411</v>
-      </c>
-      <c r="N4" s="15">
-        <f>SQRT($D$23^2-M4^2)</f>
-        <v>59.896808142659459</v>
-      </c>
-      <c r="O4" s="14">
-        <f>DEGREES(ATAN2(P4-$D$7,Q4-$D$8))</f>
-        <v>17.767431468956719</v>
-      </c>
-      <c r="P4" s="14">
-        <f>$D$7+M4*(J4-$D$7)/L4-$D$35*N4*(K4-$D$8)/L4</f>
-        <v>254.56002414514376</v>
-      </c>
-      <c r="Q4" s="14">
-        <f>$D$8+M4*(K4-$D$8)/L4+$D$35*N4*(J4-$D$7)/L4</f>
-        <v>85.935659202755687</v>
-      </c>
-      <c r="R4" s="13">
-        <f>-DEGREES(ATAN((J4-P4)/(K4-Q4)))</f>
-        <v>10.078444542415202</v>
+      <c r="T4" s="8">
+        <f>AC4-H4</f>
+        <v>-4.481455409386534</v>
+      </c>
+      <c r="U4" s="9">
+        <f t="shared" ref="U4:U44" si="0">$D$5+$D$22*COS(RADIANS(S4))</f>
+        <v>202.93816910511799</v>
+      </c>
+      <c r="V4" s="9">
+        <f t="shared" ref="V4:V44" si="1">$D$6+$D$22*SIN(RADIANS(S4))</f>
+        <v>137.46642952412375</v>
+      </c>
+      <c r="W4" s="9">
+        <f>SQRT((U4-$D$7)^2+(V4-$D$8)^2)</f>
+        <v>163.28755891855951</v>
+      </c>
+      <c r="X4" s="9">
+        <f>($D$23^2-$D$27^2+W4^2)/(2*W4)</f>
+        <v>115.32668853346802</v>
+      </c>
+      <c r="Y4" s="10">
+        <f>SQRT($D$23^2-X4^2)</f>
+        <v>46.901544877588584</v>
+      </c>
+      <c r="Z4" s="9">
+        <f>DEGREES(ATAN2(AA4-$D$7,AB4-$D$8))</f>
+        <v>19.027538152840954</v>
+      </c>
+      <c r="AA4" s="9">
+        <f>$D$7+X4*(U4-$D$7)/W4-$D$35*Y4*(V4-$D$8)/W4</f>
+        <v>197.69661835661304</v>
+      </c>
+      <c r="AB4" s="9">
+        <f>$D$8+X4*(V4-$D$8)/W4+$D$35*Y4*(U4-$D$7)/W4</f>
+        <v>70.589481733791331</v>
+      </c>
+      <c r="AC4" s="8">
+        <f>-DEGREES(ATAN((U4-AA4)/(V4-AB4)))</f>
+        <v>-4.481455409386534</v>
       </c>
     </row>
-    <row r="5" spans="3:18" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="5" spans="3:29" ht="15.75" x14ac:dyDescent="0.3">
       <c r="C5" s="2" t="s">
         <v>8</v>
       </c>
@@ -2494,51 +2560,51 @@
       <c r="F5" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="H5" s="11">
+      <c r="S5" s="6">
         <v>19</v>
       </c>
-      <c r="I5" s="13">
-        <f>R5-5</f>
-        <v>4.9929530523627381</v>
-      </c>
-      <c r="J5" s="14">
-        <f>$D$5+$D$22*COS(RADIANS(H5))</f>
-        <v>243.70638191868042</v>
-      </c>
-      <c r="K5" s="14">
-        <f>$D$6+$D$22*SIN(RADIANS(H5))</f>
-        <v>149.48207550055236</v>
-      </c>
-      <c r="L5" s="14">
-        <f t="shared" ref="L5:L44" si="0">SQRT((J5-$D$7)^2+(K5-$D$8)^2)</f>
-        <v>202.67152204200903</v>
-      </c>
-      <c r="M5" s="14">
-        <f t="shared" ref="M5:M44" si="1">($D$23^2-$D$27^2+L5^2)/(2*L5)</f>
-        <v>173.12680424899253</v>
-      </c>
-      <c r="N5" s="15">
-        <f t="shared" ref="N5:N44" si="2">SQRT($D$23^2-M5^2)</f>
-        <v>60.225490039774819</v>
-      </c>
-      <c r="O5" s="14">
-        <f t="shared" ref="O5:O44" si="3">DEGREES(ATAN2(P5-$D$7,Q5-$D$8))</f>
-        <v>16.942845540226465</v>
-      </c>
-      <c r="P5" s="14">
-        <f t="shared" ref="P5:P44" si="4">$D$7+M5*(J5-$D$7)/L5-$D$35*N5*(K5-$D$8)/L5</f>
-        <v>255.34693047487045</v>
-      </c>
-      <c r="Q5" s="14">
-        <f t="shared" ref="Q5:Q44" si="5">$D$8+M5*(K5-$D$8)/L5+$D$35*N5*(J5-$D$7)/L5</f>
-        <v>83.417730886297818</v>
-      </c>
-      <c r="R5" s="13">
-        <f>-DEGREES(ATAN((J5-P5)/(K5-Q5)))</f>
-        <v>9.9929530523627381</v>
+      <c r="T5" s="8">
+        <f>AC5-H4</f>
+        <v>-4.5096282411695068</v>
+      </c>
+      <c r="U5" s="9">
+        <f t="shared" si="0"/>
+        <v>203.5763704791799</v>
+      </c>
+      <c r="V5" s="9">
+        <f t="shared" si="1"/>
+        <v>135.66420444030217</v>
+      </c>
+      <c r="W5" s="9">
+        <f t="shared" ref="W5:W44" si="2">SQRT((U5-$D$7)^2+(V5-$D$8)^2)</f>
+        <v>162.59164628236439</v>
+      </c>
+      <c r="X5" s="9">
+        <f t="shared" ref="X5:X44" si="3">($D$23^2-$D$27^2+W5^2)/(2*W5)</f>
+        <v>115.12289929027561</v>
+      </c>
+      <c r="Y5" s="10">
+        <f t="shared" ref="Y5:Y44" si="4">SQRT($D$23^2-X5^2)</f>
+        <v>47.399557582334666</v>
+      </c>
+      <c r="Z5" s="9">
+        <f t="shared" ref="Z5:Z44" si="5">DEGREES(ATAN2(AA5-$D$7,AB5-$D$8))</f>
+        <v>18.15372127701399</v>
+      </c>
+      <c r="AA5" s="9">
+        <f t="shared" ref="AA5:AA44" si="6">$D$7+X5*(U5-$D$7)/W5-$D$35*Y5*(V5-$D$8)/W5</f>
+        <v>198.30193639031026</v>
+      </c>
+      <c r="AB5" s="9">
+        <f t="shared" ref="AB5:AB44" si="7">$D$8+X5*(V5-$D$8)/W5+$D$35*Y5*(U5-$D$7)/W5</f>
+        <v>68.78984205050314</v>
+      </c>
+      <c r="AC5" s="8">
+        <f t="shared" ref="AC5:AC44" si="8">-DEGREES(ATAN((U5-AA5)/(V5-AB5)))</f>
+        <v>-4.5096282411695068</v>
       </c>
     </row>
-    <row r="6" spans="3:18" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="6" spans="3:29" ht="15.75" x14ac:dyDescent="0.3">
       <c r="C6" s="2" t="s">
         <v>9</v>
       </c>
@@ -2551,51 +2617,51 @@
       <c r="F6" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="H6" s="11">
+      <c r="S6" s="6">
         <v>18</v>
       </c>
-      <c r="I6" s="13">
-        <f>R6-5</f>
-        <v>4.9145587013259746</v>
-      </c>
-      <c r="J6" s="14">
-        <f>$D$5+$D$22*COS(RADIANS(H6))</f>
-        <v>244.54807603365271</v>
-      </c>
-      <c r="K6" s="14">
-        <f>$D$6+$D$22*SIN(RADIANS(H6))</f>
-        <v>146.96651695590549</v>
-      </c>
-      <c r="L6" s="14">
+      <c r="T6" s="8">
+        <f>AC6-H4</f>
+        <v>-4.5337589113301595</v>
+      </c>
+      <c r="U6" s="9">
         <f t="shared" si="0"/>
-        <v>201.88421289237274</v>
-      </c>
-      <c r="M6" s="14">
+        <v>204.18302148742703</v>
+      </c>
+      <c r="V6" s="9">
         <f t="shared" si="1"/>
-        <v>173.01312077436864</v>
-      </c>
-      <c r="N6" s="15">
+        <v>133.85111569432115</v>
+      </c>
+      <c r="W6" s="9">
         <f t="shared" si="2"/>
-        <v>60.55130089365317</v>
-      </c>
-      <c r="O6" s="14">
+        <v>161.88414702095457</v>
+      </c>
+      <c r="X6" s="9">
         <f t="shared" si="3"/>
-        <v>16.117468445746898</v>
-      </c>
-      <c r="P6" s="14">
+        <v>114.91698767726145</v>
+      </c>
+      <c r="Y6" s="10">
         <f t="shared" si="4"/>
-        <v>256.09822187350994</v>
-      </c>
-      <c r="Q6" s="14">
+        <v>47.896617241556235</v>
+      </c>
+      <c r="Z6" s="9">
         <f t="shared" si="5"/>
-        <v>80.886307126653065</v>
-      </c>
-      <c r="R6" s="13">
-        <f>-DEGREES(ATAN((J6-P6)/(K6-Q6)))</f>
-        <v>9.9145587013259746</v>
+        <v>17.27884422564712</v>
+      </c>
+      <c r="AA6" s="9">
+        <f t="shared" si="6"/>
+        <v>198.88042308444278</v>
+      </c>
+      <c r="AB6" s="9">
+        <f t="shared" si="7"/>
+        <v>66.97898061417979</v>
+      </c>
+      <c r="AC6" s="8">
+        <f t="shared" si="8"/>
+        <v>-4.5337589113301595</v>
       </c>
     </row>
-    <row r="7" spans="3:18" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="7" spans="3:29" ht="15.75" x14ac:dyDescent="0.3">
       <c r="C7" s="2" t="s">
         <v>10</v>
       </c>
@@ -2608,51 +2674,51 @@
       <c r="F7" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="H7" s="11">
+      <c r="S7" s="6">
         <v>17</v>
       </c>
-      <c r="I7" s="13">
-        <f>R7-5</f>
-        <v>4.8431988789515419</v>
-      </c>
-      <c r="J7" s="14">
-        <f>$D$5+$D$22*COS(RADIANS(H7))</f>
-        <v>245.34573940439648</v>
-      </c>
-      <c r="K7" s="14">
-        <f>$D$6+$D$22*SIN(RADIANS(H7))</f>
-        <v>144.43665195521902</v>
-      </c>
-      <c r="L7" s="14">
+      <c r="T7" s="8">
+        <f>AC7-H4</f>
+        <v>-4.5539317551658343</v>
+      </c>
+      <c r="U7" s="9">
         <f t="shared" si="0"/>
-        <v>201.08446198029952</v>
-      </c>
-      <c r="M7" s="14">
+        <v>204.75793733808553</v>
+      </c>
+      <c r="V7" s="9">
         <f t="shared" si="1"/>
-        <v>172.89988536438719</v>
-      </c>
-      <c r="N7" s="15">
+        <v>132.02771557057653</v>
+      </c>
+      <c r="W7" s="9">
         <f t="shared" si="2"/>
-        <v>60.873883077899364</v>
-      </c>
-      <c r="O7" s="14">
+        <v>161.16512548750779</v>
+      </c>
+      <c r="X7" s="9">
         <f t="shared" si="3"/>
-        <v>15.291373412183672</v>
-      </c>
-      <c r="P7" s="14">
+        <v>114.70905247509666</v>
+      </c>
+      <c r="Y7" s="10">
         <f t="shared" si="4"/>
-        <v>256.81357579454135</v>
-      </c>
-      <c r="Q7" s="14">
+        <v>48.392491982388364</v>
+      </c>
+      <c r="Z7" s="9">
         <f t="shared" si="5"/>
-        <v>78.342108091683173</v>
-      </c>
-      <c r="R7" s="13">
-        <f>-DEGREES(ATAN((J7-P7)/(K7-Q7)))</f>
-        <v>9.8431988789515419</v>
+        <v>16.402985706360017</v>
+      </c>
+      <c r="AA7" s="9">
+        <f t="shared" si="6"/>
+        <v>199.43179475277836</v>
+      </c>
+      <c r="AB7" s="9">
+        <f t="shared" si="7"/>
+        <v>65.157451587540137</v>
+      </c>
+      <c r="AC7" s="8">
+        <f t="shared" si="8"/>
+        <v>-4.5539317551658343</v>
       </c>
     </row>
-    <row r="8" spans="3:18" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="8" spans="3:29" ht="15.75" x14ac:dyDescent="0.3">
       <c r="C8" s="2" t="s">
         <v>11</v>
       </c>
@@ -2665,56 +2731,56 @@
       <c r="F8" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="H8" s="11">
+      <c r="S8" s="6">
         <v>16</v>
       </c>
-      <c r="I8" s="13">
-        <f>R8-5</f>
-        <v>4.7788169483417331</v>
-      </c>
-      <c r="J8" s="14">
-        <f>$D$5+$D$22*COS(RADIANS(H8))</f>
-        <v>246.09912905492189</v>
-      </c>
-      <c r="K8" s="14">
-        <f>$D$6+$D$22*SIN(RADIANS(H8))</f>
-        <v>141.89325111987944</v>
-      </c>
-      <c r="L8" s="14">
+      <c r="T8" s="8">
+        <f>AC8-H4</f>
+        <v>-4.5702252042057925</v>
+      </c>
+      <c r="U8" s="9">
         <f t="shared" si="0"/>
-        <v>200.27236534025354</v>
-      </c>
-      <c r="M8" s="14">
+        <v>205.30094290621787</v>
+      </c>
+      <c r="V8" s="9">
         <f t="shared" si="1"/>
-        <v>172.78724451423199</v>
-      </c>
-      <c r="N8" s="15">
+        <v>130.19455949440965</v>
+      </c>
+      <c r="W8" s="9">
         <f t="shared" si="2"/>
-        <v>61.192876490478859</v>
-      </c>
-      <c r="O8" s="14">
+        <v>160.43464727254542</v>
+      </c>
+      <c r="X8" s="9">
         <f t="shared" si="3"/>
-        <v>14.464633739732029</v>
-      </c>
-      <c r="P8" s="14">
+        <v>114.49919537347066</v>
+      </c>
+      <c r="Y8" s="10">
         <f t="shared" si="4"/>
-        <v>257.49268932395222</v>
-      </c>
-      <c r="Q8" s="14">
+        <v>48.88695387143482</v>
+      </c>
+      <c r="Z8" s="9">
         <f t="shared" si="5"/>
-        <v>75.785862845980887</v>
-      </c>
-      <c r="R8" s="13">
-        <f>-DEGREES(ATAN((J8-P8)/(K8-Q8)))</f>
-        <v>9.7788169483417331</v>
+        <v>15.526222402889298</v>
+      </c>
+      <c r="AA8" s="9">
+        <f t="shared" si="6"/>
+        <v>199.9557843498585</v>
+      </c>
+      <c r="AB8" s="9">
+        <f t="shared" si="7"/>
+        <v>63.325812833451621</v>
+      </c>
+      <c r="AC8" s="8">
+        <f t="shared" si="8"/>
+        <v>-4.5702252042057925</v>
       </c>
     </row>
-    <row r="9" spans="3:18" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="9" spans="3:29" ht="15.75" x14ac:dyDescent="0.3">
       <c r="C9" s="2" t="s">
         <v>30</v>
       </c>
       <c r="D9" s="2">
-        <v>160</v>
+        <v>170</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>21</v>
@@ -2722,56 +2788,56 @@
       <c r="F9" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="H9" s="11">
+      <c r="S9" s="6">
         <v>15</v>
       </c>
-      <c r="I9" s="13">
-        <f>R9-5</f>
-        <v>4.7213623345594122</v>
-      </c>
-      <c r="J9" s="14">
-        <f>$D$5+$D$22*COS(RADIANS(H9))</f>
-        <v>246.80801549544313</v>
-      </c>
-      <c r="K9" s="14">
-        <f>$D$6+$D$22*SIN(RADIANS(H9))</f>
-        <v>139.33708919441972</v>
-      </c>
-      <c r="L9" s="14">
+      <c r="T9" s="8">
+        <f>AC9-H4</f>
+        <v>-4.5827119694154002</v>
+      </c>
+      <c r="U9" s="9">
         <f t="shared" si="0"/>
-        <v>199.44802106573152</v>
-      </c>
-      <c r="M9" s="14">
+        <v>205.81187278706787</v>
+      </c>
+      <c r="V9" s="9">
         <f t="shared" si="1"/>
-        <v>172.67534854190419</v>
-      </c>
-      <c r="N9" s="15">
+        <v>128.35220586291953</v>
+      </c>
+      <c r="W9" s="9">
         <f t="shared" si="2"/>
-        <v>61.507918237670026</v>
-      </c>
-      <c r="O9" s="14">
+        <v>159.69277921149549</v>
+      </c>
+      <c r="X9" s="9">
         <f t="shared" si="3"/>
-        <v>13.637322868824969</v>
-      </c>
-      <c r="P9" s="14">
+        <v>114.28752105299905</v>
+      </c>
+      <c r="Y9" s="10">
         <f t="shared" si="4"/>
-        <v>258.13527939725759</v>
-      </c>
-      <c r="Q9" s="14">
+        <v>49.379778569372895</v>
+      </c>
+      <c r="Z9" s="9">
         <f t="shared" si="5"/>
-        <v>73.218309014363086</v>
-      </c>
-      <c r="R9" s="13">
-        <f>-DEGREES(ATAN((J9-P9)/(K9-Q9)))</f>
-        <v>9.7213623345594122</v>
+        <v>14.648629120573638</v>
+      </c>
+      <c r="AA9" s="9">
+        <f t="shared" si="6"/>
+        <v>200.45214130636751</v>
+      </c>
+      <c r="AB9" s="9">
+        <f t="shared" si="7"/>
+        <v>61.48462568795884</v>
+      </c>
+      <c r="AC9" s="8">
+        <f t="shared" si="8"/>
+        <v>-4.5827119694154002</v>
       </c>
     </row>
-    <row r="10" spans="3:18" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="10" spans="3:29" ht="15.75" x14ac:dyDescent="0.3">
       <c r="C10" s="2" t="s">
         <v>32</v>
       </c>
       <c r="D10" s="2">
-        <v>190</v>
+        <v>180</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>21</v>
@@ -2779,51 +2845,51 @@
       <c r="F10" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="H10" s="11">
+      <c r="S10" s="6">
         <v>14</v>
       </c>
-      <c r="I10" s="13">
-        <f>R10-5</f>
-        <v>4.6707906185819752</v>
-      </c>
-      <c r="J10" s="14">
-        <f>$D$5+$D$22*COS(RADIANS(H10))</f>
-        <v>247.47218279228326</v>
-      </c>
-      <c r="K10" s="14">
-        <f>$D$6+$D$22*SIN(RADIANS(H10))</f>
-        <v>136.76894481052446</v>
-      </c>
-      <c r="L10" s="14">
+      <c r="T10" s="8">
+        <f>AC10-H4</f>
+        <v>-4.5914592125202569</v>
+      </c>
+      <c r="U10" s="9">
         <f t="shared" si="0"/>
-        <v>198.61152933594957</v>
-      </c>
-      <c r="M10" s="14">
+        <v>206.29057134644427</v>
+      </c>
+      <c r="V10" s="9">
         <f t="shared" si="1"/>
-        <v>172.56435166263412</v>
-      </c>
-      <c r="N10" s="15">
+        <v>126.50121587486956</v>
+      </c>
+      <c r="W10" s="9">
         <f t="shared" si="2"/>
-        <v>61.818642295465658</v>
-      </c>
-      <c r="O10" s="14">
+        <v>158.93958939276112</v>
+      </c>
+      <c r="X10" s="9">
         <f t="shared" si="3"/>
-        <v>12.809514452223082</v>
-      </c>
-      <c r="P10" s="14">
+        <v>114.07413727089647</v>
+      </c>
+      <c r="Y10" s="10">
         <f t="shared" si="4"/>
-        <v>258.74108301404118</v>
-      </c>
-      <c r="Q10" s="14">
+        <v>49.870744990431696</v>
+      </c>
+      <c r="Z10" s="9">
         <f t="shared" si="5"/>
-        <v>70.640192457315322</v>
-      </c>
-      <c r="R10" s="13">
-        <f>-DEGREES(ATAN((J10-P10)/(K10-Q10)))</f>
-        <v>9.6707906185819752</v>
+        <v>13.770278928452155</v>
+      </c>
+      <c r="AA10" s="9">
+        <f t="shared" si="6"/>
+        <v>200.92063137563241</v>
+      </c>
+      <c r="AB10" s="9">
+        <f t="shared" si="7"/>
+        <v>59.634454739684642</v>
+      </c>
+      <c r="AC10" s="8">
+        <f t="shared" si="8"/>
+        <v>-4.5914592125202569</v>
       </c>
     </row>
-    <row r="11" spans="3:18" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="11" spans="3:29" ht="15.75" x14ac:dyDescent="0.3">
       <c r="C11" s="2" t="s">
         <v>16</v>
       </c>
@@ -2836,51 +2902,51 @@
       <c r="F11" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="H11" s="11">
+      <c r="S11" s="6">
         <v>13</v>
       </c>
-      <c r="I11" s="13">
-        <f>R11-5</f>
-        <v>4.6270636378975958</v>
-      </c>
-      <c r="J11" s="14">
-        <f>$D$5+$D$22*COS(RADIANS(H11))</f>
-        <v>248.09142863364977</v>
-      </c>
-      <c r="K11" s="14">
-        <f>$D$6+$D$22*SIN(RADIANS(H11))</f>
-        <v>134.18960024985114</v>
-      </c>
-      <c r="L11" s="14">
+      <c r="T11" s="8">
+        <f>AC11-H4</f>
+        <v>-4.5965287054464969</v>
+      </c>
+      <c r="U11" s="9">
         <f t="shared" si="0"/>
-        <v>197.76299244379661</v>
-      </c>
-      <c r="M11" s="14">
+        <v>206.73689276812871</v>
+      </c>
+      <c r="V11" s="9">
         <f t="shared" si="1"/>
-        <v>172.45441206526596</v>
-      </c>
-      <c r="N11" s="15">
+        <v>124.64215335974107</v>
+      </c>
+      <c r="W11" s="9">
         <f t="shared" si="2"/>
-        <v>62.124679147851104</v>
-      </c>
-      <c r="O11" s="14">
+        <v>158.17514716632604</v>
+      </c>
+      <c r="X11" s="9">
         <f t="shared" si="3"/>
-        <v>11.981282432580343</v>
-      </c>
-      <c r="P11" s="14">
+        <v>113.85915495059858</v>
+      </c>
+      <c r="Y11" s="10">
         <f t="shared" si="4"/>
-        <v>259.30985745156227</v>
-      </c>
-      <c r="Q11" s="14">
+        <v>50.359634966266221</v>
+      </c>
+      <c r="Z11" s="9">
         <f t="shared" si="5"/>
-        <v>68.052266958755823</v>
-      </c>
-      <c r="R11" s="13">
-        <f>-DEGREES(ATAN((J11-P11)/(K11-Q11)))</f>
-        <v>9.6270636378975958</v>
+        <v>12.891243298134027</v>
+      </c>
+      <c r="AA11" s="9">
+        <f t="shared" si="6"/>
+        <v>201.36103649125238</v>
+      </c>
+      <c r="AB11" s="9">
+        <f t="shared" si="7"/>
+        <v>57.775867615052285</v>
+      </c>
+      <c r="AC11" s="8">
+        <f t="shared" si="8"/>
+        <v>-4.5965287054464969</v>
       </c>
     </row>
-    <row r="12" spans="3:18" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="12" spans="3:29" ht="15.75" x14ac:dyDescent="0.3">
       <c r="C12" s="2" t="s">
         <v>17</v>
       </c>
@@ -2893,56 +2959,56 @@
       <c r="F12" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="H12" s="11">
+      <c r="S12" s="6">
         <v>12</v>
       </c>
-      <c r="I12" s="13">
-        <f>R12-5</f>
-        <v>4.5901495949651991</v>
-      </c>
-      <c r="J12" s="14">
-        <f>$D$5+$D$22*COS(RADIANS(H12))</f>
-        <v>248.66556439126057</v>
-      </c>
-      <c r="K12" s="14">
-        <f>$D$6+$D$22*SIN(RADIANS(H12))</f>
-        <v>131.59984120573961</v>
-      </c>
-      <c r="L12" s="14">
+      <c r="T12" s="8">
+        <f>AC12-H4</f>
+        <v>-4.5979769778990534</v>
+      </c>
+      <c r="U12" s="9">
         <f t="shared" si="0"/>
-        <v>196.90251482511331</v>
-      </c>
-      <c r="M12" s="14">
+        <v>207.15070109829242</v>
+      </c>
+      <c r="V12" s="9">
         <f t="shared" si="1"/>
-        <v>172.34569199061755</v>
-      </c>
-      <c r="N12" s="15">
+        <v>122.7755846059853</v>
+      </c>
+      <c r="W12" s="9">
         <f t="shared" si="2"/>
-        <v>62.425655401246502</v>
-      </c>
-      <c r="O12" s="14">
+        <v>157.39952315292965</v>
+      </c>
+      <c r="X12" s="9">
         <f t="shared" si="3"/>
-        <v>11.152701125618671</v>
-      </c>
-      <c r="P12" s="14">
+        <v>113.64268827552598</v>
+      </c>
+      <c r="Y12" s="10">
         <f t="shared" si="4"/>
-        <v>259.84138047897761</v>
-      </c>
-      <c r="Q12" s="14">
+        <v>50.84623291367442</v>
+      </c>
+      <c r="Z12" s="9">
         <f t="shared" si="5"/>
-        <v>65.455293926515495</v>
-      </c>
-      <c r="R12" s="13">
-        <f>-DEGREES(ATAN((J12-P12)/(K12-Q12)))</f>
-        <v>9.5901495949651991</v>
+        <v>12.011592239625786</v>
+      </c>
+      <c r="AA12" s="9">
+        <f t="shared" si="6"/>
+        <v>201.77315463582019</v>
+      </c>
+      <c r="AB12" s="9">
+        <f t="shared" si="7"/>
+        <v>55.909434768837123</v>
+      </c>
+      <c r="AC12" s="8">
+        <f t="shared" si="8"/>
+        <v>-4.5979769778990534</v>
       </c>
     </row>
-    <row r="13" spans="3:18" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="13" spans="3:29" ht="15.75" x14ac:dyDescent="0.3">
       <c r="C13" s="2" t="s">
         <v>19</v>
       </c>
       <c r="D13" s="2">
-        <v>150</v>
+        <v>310</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>21</v>
@@ -2950,51 +3016,51 @@
       <c r="F13" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="H13" s="11">
+      <c r="S13" s="6">
         <v>11</v>
       </c>
-      <c r="I13" s="13">
-        <f>R13-5</f>
-        <v>4.5600231747982534</v>
-      </c>
-      <c r="J13" s="14">
-        <f>$D$5+$D$22*COS(RADIANS(H13))</f>
-        <v>249.19441517780214</v>
-      </c>
-      <c r="K13" s="14">
-        <f>$D$6+$D$22*SIN(RADIANS(H13))</f>
-        <v>129.00045654388231</v>
-      </c>
-      <c r="L13" s="14">
+      <c r="T13" s="8">
+        <f>AC13-H4</f>
+        <v>-4.5958554531206639</v>
+      </c>
+      <c r="U13" s="9">
         <f t="shared" si="0"/>
-        <v>196.0302030893597</v>
-      </c>
-      <c r="M13" s="14">
+        <v>207.53187028690948</v>
+      </c>
+      <c r="V13" s="9">
         <f t="shared" si="1"/>
-        <v>172.23835781181452</v>
-      </c>
-      <c r="N13" s="15">
+        <v>120.9020781885265</v>
+      </c>
+      <c r="W13" s="9">
         <f t="shared" si="2"/>
-        <v>62.721193374244272</v>
-      </c>
-      <c r="O13" s="14">
+        <v>156.61278925384764</v>
+      </c>
+      <c r="X13" s="9">
         <f t="shared" si="3"/>
-        <v>10.323845309088249</v>
-      </c>
-      <c r="P13" s="14">
+        <v>113.42485478719375</v>
+      </c>
+      <c r="Y13" s="10">
         <f t="shared" si="4"/>
-        <v>260.33545057374437</v>
-      </c>
-      <c r="Q13" s="14">
+        <v>51.330325505533381</v>
+      </c>
+      <c r="Z13" s="9">
         <f t="shared" si="5"/>
-        <v>62.850042105979064</v>
-      </c>
-      <c r="R13" s="13">
-        <f>-DEGREES(ATAN((J13-P13)/(K13-Q13)))</f>
-        <v>9.5600231747982534</v>
+        <v>11.131394434329703</v>
+      </c>
+      <c r="AA13" s="9">
+        <f t="shared" si="6"/>
+        <v>202.15679972067437</v>
+      </c>
+      <c r="AB13" s="9">
+        <f t="shared" si="7"/>
+        <v>54.035729279617215</v>
+      </c>
+      <c r="AC13" s="8">
+        <f t="shared" si="8"/>
+        <v>-4.5958554531206639</v>
       </c>
     </row>
-    <row r="14" spans="3:18" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="14" spans="3:29" ht="15.75" x14ac:dyDescent="0.3">
       <c r="C14" s="2" t="s">
         <v>18</v>
       </c>
@@ -3007,56 +3073,56 @@
       <c r="F14" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="H14" s="11">
+      <c r="S14" s="6">
         <v>10</v>
       </c>
-      <c r="I14" s="13">
-        <f>R14-5</f>
-        <v>4.5366656729775681</v>
-      </c>
-      <c r="J14" s="14">
-        <f>$D$5+$D$22*COS(RADIANS(H14))</f>
-        <v>249.6778199002018</v>
-      </c>
-      <c r="K14" s="14">
-        <f>$D$6+$D$22*SIN(RADIANS(H14))</f>
-        <v>126.39223806202797</v>
-      </c>
-      <c r="L14" s="14">
+      <c r="T14" s="8">
+        <f>AC14-H4</f>
+        <v>-4.5902105718840218</v>
+      </c>
+      <c r="U14" s="9">
         <f t="shared" si="0"/>
-        <v>195.14616605173669</v>
-      </c>
-      <c r="M14" s="14">
+        <v>207.88028422615253</v>
+      </c>
+      <c r="V14" s="9">
         <f t="shared" si="1"/>
-        <v>172.13258011659028</v>
-      </c>
-      <c r="N14" s="15">
+        <v>119.02220479556851</v>
+      </c>
+      <c r="W14" s="9">
         <f t="shared" si="2"/>
-        <v>63.010910661611803</v>
-      </c>
-      <c r="O14" s="14">
+        <v>155.81501866131421</v>
+      </c>
+      <c r="X14" s="9">
         <f t="shared" si="3"/>
-        <v>9.4947903177358484</v>
-      </c>
-      <c r="P14" s="14">
+        <v>113.20577548788178</v>
+      </c>
+      <c r="Y14" s="10">
         <f t="shared" si="4"/>
-        <v>260.79188714179276</v>
-      </c>
-      <c r="Q14" s="14">
+        <v>51.811701344264925</v>
+      </c>
+      <c r="Z14" s="9">
         <f t="shared" si="5"/>
-        <v>60.237287307383838</v>
-      </c>
-      <c r="R14" s="13">
-        <f>-DEGREES(ATAN((J14-P14)/(K14-Q14)))</f>
-        <v>9.5366656729775681</v>
+        <v>10.250717365450708</v>
+      </c>
+      <c r="AA14" s="9">
+        <f t="shared" si="6"/>
+        <v>202.51180147660429</v>
+      </c>
+      <c r="AB14" s="9">
+        <f t="shared" si="7"/>
+        <v>52.155326649749526</v>
+      </c>
+      <c r="AC14" s="8">
+        <f t="shared" si="8"/>
+        <v>-4.5902105718840218</v>
       </c>
     </row>
-    <row r="15" spans="3:18" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="15" spans="3:29" ht="15.75" x14ac:dyDescent="0.3">
       <c r="C15" s="2" t="s">
         <v>20</v>
       </c>
       <c r="D15" s="2">
-        <v>130</v>
+        <v>290</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>21</v>
@@ -3064,56 +3130,56 @@
       <c r="F15" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="H15" s="11">
+      <c r="S15" s="6">
         <v>9</v>
       </c>
-      <c r="I15" s="13">
-        <f>R15-5</f>
-        <v>4.5200651354569228</v>
-      </c>
-      <c r="J15" s="14">
-        <f>$D$5+$D$22*COS(RADIANS(H15))</f>
-        <v>250.11563130869825</v>
-      </c>
-      <c r="K15" s="14">
-        <f>$D$6+$D$22*SIN(RADIANS(H15))</f>
-        <v>123.77598024879261</v>
-      </c>
-      <c r="L15" s="14">
+      <c r="T15" s="8">
+        <f>AC15-H4</f>
+        <v>-4.5810839047740481</v>
+      </c>
+      <c r="U15" s="9">
         <f t="shared" si="0"/>
-        <v>194.25051476683117</v>
-      </c>
-      <c r="M15" s="14">
+        <v>208.19583678576049</v>
+      </c>
+      <c r="V15" s="9">
         <f t="shared" si="1"/>
-        <v>172.02853379153788</v>
-      </c>
-      <c r="N15" s="15">
+        <v>117.13653705475755</v>
+      </c>
+      <c r="W15" s="9">
         <f t="shared" si="2"/>
-        <v>63.294419671355705</v>
-      </c>
-      <c r="O15" s="14">
+        <v>155.00628586962685</v>
+      </c>
+      <c r="X15" s="9">
         <f t="shared" si="3"/>
-        <v>8.665612144551865</v>
-      </c>
-      <c r="P15" s="14">
+        <v>112.98557494809292</v>
+      </c>
+      <c r="Y15" s="10">
         <f t="shared" si="4"/>
-        <v>261.21053074309577</v>
-      </c>
-      <c r="Q15" s="14">
+        <v>52.29015063708345</v>
+      </c>
+      <c r="Z15" s="9">
         <f t="shared" si="5"/>
-        <v>57.617812147335911</v>
-      </c>
-      <c r="R15" s="13">
-        <f>-DEGREES(ATAN((J15-P15)/(K15-Q15)))</f>
-        <v>9.5200651354569228</v>
+        <v>9.3696274460685736</v>
+      </c>
+      <c r="AA15" s="9">
+        <f t="shared" si="6"/>
+        <v>202.83800535542721</v>
+      </c>
+      <c r="AB15" s="9">
+        <f t="shared" si="7"/>
+        <v>50.268804609547999</v>
+      </c>
+      <c r="AC15" s="8">
+        <f t="shared" si="8"/>
+        <v>-4.5810839047740481</v>
       </c>
     </row>
-    <row r="16" spans="3:18" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="16" spans="3:29" ht="15.75" x14ac:dyDescent="0.3">
       <c r="C16" s="2" t="s">
         <v>27</v>
       </c>
       <c r="D16" s="2">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>1</v>
@@ -3121,147 +3187,147 @@
       <c r="F16" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="H16" s="11">
+      <c r="S16" s="6">
         <v>8</v>
       </c>
-      <c r="I16" s="13">
-        <f>R16-5</f>
-        <v>4.5102165115946331</v>
-      </c>
-      <c r="J16" s="14">
-        <f>$D$5+$D$22*COS(RADIANS(H16))</f>
-        <v>250.50771604169532</v>
-      </c>
-      <c r="K16" s="14">
-        <f>$D$6+$D$22*SIN(RADIANS(H16))</f>
-        <v>121.15248004165036</v>
-      </c>
-      <c r="L16" s="14">
+      <c r="T16" s="8">
+        <f>AC16-H4</f>
+        <v>-4.5685122528115603</v>
+      </c>
+      <c r="U16" s="9">
         <f t="shared" si="0"/>
-        <v>193.34336256385652</v>
-      </c>
-      <c r="M16" s="14">
+        <v>208.47843184536691</v>
+      </c>
+      <c r="V16" s="9">
         <f t="shared" si="1"/>
-        <v>171.92639810829195</v>
-      </c>
-      <c r="N16" s="15">
+        <v>115.24564935875435</v>
+      </c>
+      <c r="W16" s="9">
         <f t="shared" si="2"/>
-        <v>63.571327133457743</v>
-      </c>
-      <c r="O16" s="14">
+        <v>154.18666668697489</v>
+      </c>
+      <c r="X16" s="9">
         <f t="shared" si="3"/>
-        <v>7.8363875486192649</v>
-      </c>
-      <c r="P16" s="14">
+        <v>112.76438141903819</v>
+      </c>
+      <c r="Y16" s="10">
         <f t="shared" si="4"/>
-        <v>261.59124332431145</v>
-      </c>
-      <c r="Q16" s="14">
+        <v>52.765464872221827</v>
+      </c>
+      <c r="Z16" s="9">
         <f t="shared" si="5"/>
-        <v>54.992405805178102</v>
-      </c>
-      <c r="R16" s="13">
-        <f>-DEGREES(ATAN((J16-P16)/(K16-Q16)))</f>
-        <v>9.5102165115946331</v>
+        <v>8.4881901451512096</v>
+      </c>
+      <c r="AA16" s="9">
+        <f t="shared" si="6"/>
+        <v>203.13527244235962</v>
+      </c>
+      <c r="AB16" s="9">
+        <f t="shared" si="7"/>
+        <v>48.376742925389841</v>
+      </c>
+      <c r="AC16" s="8">
+        <f t="shared" si="8"/>
+        <v>-4.5685122528115603</v>
       </c>
     </row>
-    <row r="17" spans="3:18" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="H17" s="11">
+    <row r="17" spans="3:29" ht="15.75" x14ac:dyDescent="0.3">
+      <c r="S17" s="6">
         <v>7</v>
       </c>
-      <c r="I17" s="13">
-        <f>R17-5</f>
-        <v>4.5071218219256117</v>
-      </c>
-      <c r="J17" s="14">
-        <f>$D$5+$D$22*COS(RADIANS(H17))</f>
-        <v>250.85395466638505</v>
-      </c>
-      <c r="K17" s="14">
-        <f>$D$6+$D$22*SIN(RADIANS(H17))</f>
-        <v>118.52253658417877</v>
-      </c>
-      <c r="L17" s="14">
+      <c r="T17" s="8">
+        <f>AC17-H4</f>
+        <v>-4.552527736461915</v>
+      </c>
+      <c r="U17" s="9">
         <f t="shared" si="0"/>
-        <v>192.42482508356457</v>
-      </c>
-      <c r="M17" s="14">
+        <v>208.72798332377909</v>
+      </c>
+      <c r="V17" s="9">
         <f t="shared" si="1"/>
-        <v>171.82635681161</v>
-      </c>
-      <c r="N17" s="15">
+        <v>113.35011769026855</v>
+      </c>
+      <c r="W17" s="9">
         <f t="shared" si="2"/>
-        <v>63.84123357869332</v>
-      </c>
-      <c r="O17" s="14">
+        <v>153.35623824803724</v>
+      </c>
+      <c r="X17" s="9">
         <f t="shared" si="3"/>
-        <v>7.0071941699438831</v>
-      </c>
-      <c r="P17" s="14">
+        <v>112.5423269504022</v>
+      </c>
+      <c r="Y17" s="10">
         <f t="shared" si="4"/>
-        <v>261.93390846023465</v>
-      </c>
-      <c r="Q17" s="14">
+        <v>53.237436495278153</v>
+      </c>
+      <c r="Z17" s="9">
         <f t="shared" si="5"/>
-        <v>52.361863794929121</v>
-      </c>
-      <c r="R17" s="13">
-        <f>-DEGREES(ATAN((J17-P17)/(K17-Q17)))</f>
-        <v>9.5071218219256117</v>
+        <v>7.6064701118015599</v>
+      </c>
+      <c r="AA17" s="9">
+        <f t="shared" si="6"/>
+        <v>203.40347937911491</v>
+      </c>
+      <c r="AB17" s="9">
+        <f t="shared" si="7"/>
+        <v>46.479723211521438</v>
+      </c>
+      <c r="AC17" s="8">
+        <f t="shared" si="8"/>
+        <v>-4.552527736461915</v>
       </c>
     </row>
-    <row r="18" spans="3:18" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="C18" s="7" t="s">
+    <row r="18" spans="3:29" ht="15.75" x14ac:dyDescent="0.3">
+      <c r="C18" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="D18" s="8"/>
-      <c r="E18" s="8"/>
-      <c r="F18" s="9"/>
-      <c r="H18" s="11">
+      <c r="D18" s="13"/>
+      <c r="E18" s="13"/>
+      <c r="F18" s="14"/>
+      <c r="S18" s="6">
         <v>6</v>
       </c>
-      <c r="I18" s="13">
-        <f>R18-5</f>
-        <v>4.510790342286521</v>
-      </c>
-      <c r="J18" s="14">
-        <f>$D$5+$D$22*COS(RADIANS(H18))</f>
-        <v>251.15424171512836</v>
-      </c>
-      <c r="K18" s="14">
-        <f>$D$6+$D$22*SIN(RADIANS(H18))</f>
-        <v>115.88695098263179</v>
-      </c>
-      <c r="L18" s="14">
+      <c r="T18" s="8">
+        <f>AC18-H4</f>
+        <v>-4.533157873055548</v>
+      </c>
+      <c r="U18" s="9">
         <f t="shared" si="0"/>
-        <v>191.49502031690949</v>
-      </c>
-      <c r="M18" s="14">
+        <v>208.94441520519916</v>
+      </c>
+      <c r="V18" s="9">
         <f t="shared" si="1"/>
-        <v>171.72859820931305</v>
-      </c>
-      <c r="N18" s="15">
+        <v>111.45051944660879</v>
+      </c>
+      <c r="W18" s="9">
         <f t="shared" si="2"/>
-        <v>64.103732785730315</v>
-      </c>
-      <c r="O18" s="14">
+        <v>152.51507902739715</v>
+      </c>
+      <c r="X18" s="9">
         <f t="shared" si="3"/>
-        <v>6.1781106517050066</v>
-      </c>
-      <c r="P18" s="14">
+        <v>112.31954751365511</v>
+      </c>
+      <c r="Y18" s="10">
         <f t="shared" si="4"/>
-        <v>262.23843160587455</v>
-      </c>
-      <c r="Q18" s="14">
+        <v>53.705858584774269</v>
+      </c>
+      <c r="Z18" s="9">
         <f t="shared" si="5"/>
-        <v>49.726987753607297</v>
-      </c>
-      <c r="R18" s="13">
-        <f>-DEGREES(ATAN((J18-P18)/(K18-Q18)))</f>
-        <v>9.510790342286521</v>
+        <v>6.7245312980453704</v>
+      </c>
+      <c r="AA18" s="9">
+        <f t="shared" si="6"/>
+        <v>203.64251829767838</v>
+      </c>
+      <c r="AB18" s="9">
+        <f t="shared" si="7"/>
+        <v>44.578328745376176</v>
+      </c>
+      <c r="AC18" s="8">
+        <f t="shared" si="8"/>
+        <v>-4.533157873055548</v>
       </c>
     </row>
-    <row r="19" spans="3:18" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="19" spans="3:29" ht="15.75" x14ac:dyDescent="0.3">
       <c r="C19" s="2" t="s">
         <v>3</v>
       </c>
@@ -3274,57 +3340,57 @@
       <c r="F19" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="H19" s="11">
+      <c r="S19" s="6">
         <v>5</v>
       </c>
-      <c r="I19" s="13">
-        <f>R19-5</f>
-        <v>4.521238806021131</v>
-      </c>
-      <c r="J19" s="14">
-        <f>$D$5+$D$22*COS(RADIANS(H19))</f>
-        <v>251.40848571758124</v>
-      </c>
-      <c r="K19" s="14">
-        <f>$D$6+$D$22*SIN(RADIANS(H19))</f>
-        <v>113.24652606191513</v>
-      </c>
-      <c r="L19" s="14">
+      <c r="T19" s="8">
+        <f>AC19-H4</f>
+        <v>-4.5104256426280429</v>
+      </c>
+      <c r="U19" s="9">
         <f t="shared" si="0"/>
-        <v>190.55406864554578</v>
-      </c>
-      <c r="M19" s="14">
+        <v>209.12766156237956</v>
+      </c>
+      <c r="V19" s="9">
         <f t="shared" si="1"/>
-        <v>171.63331526403582</v>
-      </c>
-      <c r="N19" s="15">
+        <v>109.54743326380193</v>
+      </c>
+      <c r="W19" s="9">
         <f t="shared" si="2"/>
-        <v>64.35841119446691</v>
-      </c>
-      <c r="O19" s="14">
+        <v>151.66326885382452</v>
+      </c>
+      <c r="X19" s="9">
         <f t="shared" si="3"/>
-        <v>5.3492167704336646</v>
-      </c>
-      <c r="P19" s="14">
+        <v>112.09618313119336</v>
+      </c>
+      <c r="Y19" s="10">
         <f t="shared" si="4"/>
-        <v>262.50474036106687</v>
-      </c>
-      <c r="Q19" s="14">
+        <v>54.170524525963032</v>
+      </c>
+      <c r="Z19" s="9">
         <f t="shared" si="5"/>
-        <v>47.08858524687065</v>
-      </c>
-      <c r="R19" s="13">
-        <f>-DEGREES(ATAN((J19-P19)/(K19-Q19)))</f>
-        <v>9.521238806021131</v>
+        <v>5.8424370804836787</v>
+      </c>
+      <c r="AA19" s="9">
+        <f t="shared" si="6"/>
+        <v>203.85229676473358</v>
+      </c>
+      <c r="AB19" s="9">
+        <f t="shared" si="7"/>
+        <v>42.673144286260168</v>
+      </c>
+      <c r="AC19" s="8">
+        <f t="shared" si="8"/>
+        <v>-4.5104256426280429</v>
       </c>
     </row>
-    <row r="20" spans="3:18" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="20" spans="3:29" ht="15.75" x14ac:dyDescent="0.3">
       <c r="C20" s="2" t="s">
         <v>40</v>
       </c>
       <c r="D20" s="2">
         <f>D13-D12</f>
-        <v>100</v>
+        <v>260</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>21</v>
@@ -3332,57 +3398,57 @@
       <c r="F20" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="H20" s="11">
+      <c r="S20" s="6">
         <v>4</v>
       </c>
-      <c r="I20" s="13">
-        <f>R20-5</f>
-        <v>4.5384916261219512</v>
-      </c>
-      <c r="J20" s="14">
-        <f>$D$5+$D$22*COS(RADIANS(H20))</f>
-        <v>251.61660922855759</v>
-      </c>
-      <c r="K20" s="14">
-        <f>$D$6+$D$22*SIN(RADIANS(H20))</f>
-        <v>110.60206612103805</v>
-      </c>
-      <c r="L20" s="14">
+      <c r="T20" s="8">
+        <f>AC20-H4</f>
+        <v>-4.4843495421615902</v>
+      </c>
+      <c r="U20" s="9">
         <f t="shared" si="0"/>
-        <v>189.60209288424966</v>
-      </c>
-      <c r="M20" s="14">
+        <v>209.2776665767046</v>
+      </c>
+      <c r="V20" s="9">
         <f t="shared" si="1"/>
-        <v>171.54070568672313</v>
-      </c>
-      <c r="N20" s="15">
+        <v>107.64143884033486</v>
+      </c>
+      <c r="W20" s="9">
         <f t="shared" si="2"/>
-        <v>64.60484728331943</v>
-      </c>
-      <c r="O20" s="14">
+        <v>150.80088892548036</v>
+      </c>
+      <c r="X20" s="9">
         <f t="shared" si="3"/>
-        <v>4.5205935746955488</v>
-      </c>
-      <c r="P20" s="14">
+        <v>111.8723780116059</v>
+      </c>
+      <c r="Y20" s="10">
         <f t="shared" si="4"/>
-        <v>262.7327847496411</v>
-      </c>
-      <c r="Q20" s="14">
+        <v>54.631227681870342</v>
+      </c>
+      <c r="Z20" s="9">
         <f t="shared" si="5"/>
-        <v>44.447469593022966</v>
-      </c>
-      <c r="R20" s="13">
-        <f>-DEGREES(ATAN((J20-P20)/(K20-Q20)))</f>
-        <v>9.5384916261219512</v>
+        <v>4.9602503811467935</v>
+      </c>
+      <c r="AA20" s="9">
+        <f t="shared" si="6"/>
+        <v>204.03273773674283</v>
+      </c>
+      <c r="AB20" s="9">
+        <f t="shared" si="7"/>
+        <v>40.764755897296055</v>
+      </c>
+      <c r="AC20" s="8">
+        <f t="shared" si="8"/>
+        <v>-4.4843495421615902</v>
       </c>
     </row>
-    <row r="21" spans="3:18" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="21" spans="3:29" ht="15.75" x14ac:dyDescent="0.3">
       <c r="C21" s="2" t="s">
         <v>43</v>
       </c>
       <c r="D21" s="2">
         <f>D15-D14</f>
-        <v>100</v>
+        <v>260</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>21</v>
@@ -3390,57 +3456,57 @@
       <c r="F21" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="H21" s="11">
+      <c r="S21" s="6">
         <v>3</v>
       </c>
-      <c r="I21" s="13">
-        <f>R21-5</f>
-        <v>4.562581139320443</v>
-      </c>
-      <c r="J21" s="14">
-        <f>$D$5+$D$22*COS(RADIANS(H21))</f>
-        <v>251.77854885161986</v>
-      </c>
-      <c r="K21" s="14">
-        <f>$D$6+$D$22*SIN(RADIANS(H21))</f>
-        <v>107.95437668811599</v>
-      </c>
-      <c r="L21" s="14">
+      <c r="T21" s="8">
+        <f>AC21-H4</f>
+        <v>-4.4549436281809491</v>
+      </c>
+      <c r="U21" s="9">
         <f t="shared" si="0"/>
-        <v>188.63921832535522</v>
-      </c>
-      <c r="M21" s="14">
+        <v>209.39438455519388</v>
+      </c>
+      <c r="V21" s="9">
         <f t="shared" si="1"/>
-        <v>171.45097203179694</v>
-      </c>
-      <c r="N21" s="15">
+        <v>105.73311676057273</v>
+      </c>
+      <c r="W21" s="9">
         <f t="shared" si="2"/>
-        <v>64.842610907889721</v>
-      </c>
-      <c r="O21" s="14">
+        <v>149.9280218261014</v>
+      </c>
+      <c r="X21" s="9">
         <f t="shared" si="3"/>
-        <v>3.6923235329357627</v>
-      </c>
-      <c r="P21" s="14">
+        <v>111.64828069138034</v>
+      </c>
+      <c r="Y21" s="10">
         <f t="shared" si="4"/>
-        <v>262.92253751529819</v>
-      </c>
-      <c r="Q21" s="14">
+        <v>55.087761060500078</v>
+      </c>
+      <c r="Z21" s="9">
         <f t="shared" si="5"/>
-        <v>41.804459706582229</v>
-      </c>
-      <c r="R21" s="13">
-        <f>-DEGREES(ATAN((J21-P21)/(K21-Q21)))</f>
-        <v>9.562581139320443</v>
+        <v>4.078033787902517</v>
+      </c>
+      <c r="AA21" s="9">
+        <f t="shared" si="6"/>
+        <v>204.18377952572109</v>
+      </c>
+      <c r="AB21" s="9">
+        <f t="shared" si="7"/>
+        <v>38.853750770554271</v>
+      </c>
+      <c r="AC21" s="8">
+        <f t="shared" si="8"/>
+        <v>-4.4549436281809491</v>
       </c>
     </row>
-    <row r="22" spans="3:18" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="22" spans="3:29" ht="15.75" x14ac:dyDescent="0.3">
       <c r="C22" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D22" s="2">
         <f>SQRT((D9^2)-(D20/2)^2)</f>
-        <v>151.98684153570665</v>
+        <v>109.54451150103323</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>21</v>
@@ -3448,57 +3514,57 @@
       <c r="F22" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="H22" s="11">
+      <c r="S22" s="6">
         <v>2</v>
       </c>
-      <c r="I22" s="13">
-        <f>R22-5</f>
-        <v>4.5935478743113354</v>
-      </c>
-      <c r="J22" s="14">
-        <f>$D$5+$D$22*COS(RADIANS(H22))</f>
-        <v>251.89425525839013</v>
-      </c>
-      <c r="K22" s="14">
-        <f>$D$6+$D$22*SIN(RADIANS(H22))</f>
-        <v>105.30426427499893</v>
-      </c>
-      <c r="L22" s="14">
+      <c r="T22" s="8">
+        <f>AC22-H4</f>
+        <v>-4.4222175476229966</v>
+      </c>
+      <c r="U22" s="9">
         <f t="shared" si="0"/>
-        <v>187.66557278530195</v>
-      </c>
-      <c r="M22" s="14">
+        <v>209.47777994442043</v>
+      </c>
+      <c r="V22" s="9">
         <f t="shared" si="1"/>
-        <v>171.36432179390366</v>
-      </c>
-      <c r="N22" s="15">
+        <v>103.82304831790739</v>
+      </c>
+      <c r="W22" s="9">
         <f t="shared" si="2"/>
-        <v>65.071262598134908</v>
-      </c>
-      <c r="O22" s="14">
+        <v>149.0447515422259</v>
+      </c>
+      <c r="X22" s="9">
         <f t="shared" si="3"/>
-        <v>2.8644906912304831</v>
-      </c>
-      <c r="P22" s="14">
+        <v>111.42404418338035</v>
+      </c>
+      <c r="Y22" s="10">
         <f t="shared" si="4"/>
-        <v>263.07399443650547</v>
-      </c>
-      <c r="Q22" s="14">
+        <v>55.539916977072494</v>
+      </c>
+      <c r="Z22" s="9">
         <f t="shared" si="5"/>
-        <v>39.160379962771657</v>
-      </c>
-      <c r="R22" s="13">
-        <f>-DEGREES(ATAN((J22-P22)/(K22-Q22)))</f>
-        <v>9.5935478743113354</v>
+        <v>3.1958496747870471</v>
+      </c>
+      <c r="AA22" s="9">
+        <f t="shared" si="6"/>
+        <v>204.30537577577954</v>
+      </c>
+      <c r="AB22" s="9">
+        <f t="shared" si="7"/>
+        <v>36.940717055336805</v>
+      </c>
+      <c r="AC22" s="8">
+        <f t="shared" si="8"/>
+        <v>-4.4222175476229966</v>
       </c>
     </row>
-    <row r="23" spans="3:18" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="23" spans="3:29" ht="15.75" x14ac:dyDescent="0.3">
       <c r="C23" s="2" t="s">
         <v>13</v>
       </c>
       <c r="D23" s="2">
         <f>SQRT((D10^2)-(D21/2)^2)</f>
-        <v>183.30302779823359</v>
+        <v>124.49899597988733</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>21</v>
@@ -3506,57 +3572,57 @@
       <c r="F23" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="H23" s="11">
+      <c r="S23" s="6">
         <v>1</v>
       </c>
-      <c r="I23" s="13">
-        <f>R23-5</f>
-        <v>4.6314408465004711</v>
-      </c>
-      <c r="J23" s="14">
-        <f>$D$5+$D$22*COS(RADIANS(H23))</f>
-        <v>251.96369320357596</v>
-      </c>
-      <c r="K23" s="14">
-        <f>$D$6+$D$22*SIN(RADIANS(H23))</f>
-        <v>102.65253613160016</v>
-      </c>
-      <c r="L23" s="14">
+      <c r="T23" s="8">
+        <f>AC23-H4</f>
+        <v>-4.3861765568610096</v>
+      </c>
+      <c r="U23" s="9">
         <f t="shared" si="0"/>
-        <v>186.68128665339509</v>
-      </c>
-      <c r="M23" s="14">
+        <v>209.52782734134087</v>
+      </c>
+      <c r="V23" s="9">
         <f t="shared" si="1"/>
-        <v>171.2809675061344</v>
-      </c>
-      <c r="N23" s="15">
+        <v>101.91181533768972</v>
+      </c>
+      <c r="W23" s="9">
         <f t="shared" si="2"/>
-        <v>65.290352810828978</v>
-      </c>
-      <c r="O23" s="14">
+        <v>148.15116348152719</v>
+      </c>
+      <c r="X23" s="9">
         <f t="shared" si="3"/>
-        <v>2.0371808417857777</v>
-      </c>
-      <c r="P23" s="14">
+        <v>111.19982613244392</v>
+      </c>
+      <c r="Y23" s="10">
         <f t="shared" si="4"/>
-        <v>263.18717466289917</v>
-      </c>
-      <c r="Q23" s="14">
+        <v>55.987486710105522</v>
+      </c>
+      <c r="Z23" s="9">
         <f t="shared" si="5"/>
-        <v>36.516060084472919</v>
-      </c>
-      <c r="R23" s="13">
-        <f>-DEGREES(ATAN((J23-P23)/(K23-Q23)))</f>
-        <v>9.6314408465004711</v>
+        <v>2.3137603226416652</v>
+      </c>
+      <c r="AA23" s="9">
+        <f t="shared" si="6"/>
+        <v>204.39749545056227</v>
+      </c>
+      <c r="AB23" s="9">
+        <f t="shared" si="7"/>
+        <v>35.026243689609601</v>
+      </c>
+      <c r="AC23" s="8">
+        <f t="shared" si="8"/>
+        <v>-4.3861765568610096</v>
       </c>
     </row>
-    <row r="24" spans="3:18" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="24" spans="3:29" ht="15.75" x14ac:dyDescent="0.3">
       <c r="C24" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D24" s="2">
         <f>(D12+D13)/2</f>
-        <v>100</v>
+        <v>180</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>21</v>
@@ -3564,57 +3630,57 @@
       <c r="F24" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="H24" s="11">
+      <c r="S24" s="6">
         <v>0</v>
       </c>
-      <c r="I24" s="13">
-        <f>R24-5</f>
-        <v>4.6763178818957858</v>
-      </c>
-      <c r="J24" s="14">
-        <f>$D$5+$D$22*COS(RADIANS(H24))</f>
-        <v>251.98684153570665</v>
-      </c>
-      <c r="K24" s="14">
-        <f>$D$6+$D$22*SIN(RADIANS(H24))</f>
+      <c r="T24" s="8">
+        <f>AC24-H4</f>
+        <v>-4.346821528722181</v>
+      </c>
+      <c r="U24" s="9">
+        <f t="shared" si="0"/>
+        <v>209.54451150103324</v>
+      </c>
+      <c r="V24" s="9">
+        <f t="shared" si="1"/>
         <v>100</v>
       </c>
-      <c r="L24" s="14">
-        <f t="shared" si="0"/>
-        <v>185.68649294288551</v>
-      </c>
-      <c r="M24" s="14">
-        <f t="shared" si="1"/>
-        <v>171.20112683959297</v>
-      </c>
-      <c r="N24" s="15">
+      <c r="W24" s="9">
         <f t="shared" si="2"/>
-        <v>65.499421133729044</v>
-      </c>
-      <c r="O24" s="14">
+        <v>147.24734449232466</v>
+      </c>
+      <c r="X24" s="9">
         <f t="shared" si="3"/>
-        <v>1.2104817031324244</v>
-      </c>
-      <c r="P24" s="14">
+        <v>110.97578897847251</v>
+      </c>
+      <c r="Y24" s="10">
         <f t="shared" si="4"/>
-        <v>263.26212107589026</v>
-      </c>
-      <c r="Q24" s="14">
+        <v>56.430260150078524</v>
+      </c>
+      <c r="Z24" s="9">
         <f t="shared" si="5"/>
-        <v>33.872335053392931</v>
-      </c>
-      <c r="R24" s="13">
-        <f>-DEGREES(ATAN((J24-P24)/(K24-Q24)))</f>
-        <v>9.6763178818957858</v>
+        <v>1.4318280404579051</v>
+      </c>
+      <c r="AA24" s="9">
+        <f t="shared" si="6"/>
+        <v>204.46012283174818</v>
+      </c>
+      <c r="AB24" s="9">
+        <f t="shared" si="7"/>
+        <v>33.110920234617922</v>
+      </c>
+      <c r="AC24" s="8">
+        <f t="shared" si="8"/>
+        <v>-4.346821528722181</v>
       </c>
     </row>
-    <row r="25" spans="3:18" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="25" spans="3:29" ht="15.75" x14ac:dyDescent="0.3">
       <c r="C25" s="2" t="s">
         <v>15</v>
       </c>
       <c r="D25" s="2">
         <f>(D14+D15)/2</f>
-        <v>80</v>
+        <v>160</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>21</v>
@@ -3622,51 +3688,51 @@
       <c r="F25" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="H25" s="11">
+      <c r="S25" s="6">
         <v>-1</v>
       </c>
-      <c r="I25" s="13">
-        <f>R25-5</f>
-        <v>4.7282459730292103</v>
-      </c>
-      <c r="J25" s="14">
-        <f>$D$5+$D$22*COS(RADIANS(H25))</f>
-        <v>251.96369320357596</v>
-      </c>
-      <c r="K25" s="14">
-        <f>$D$6+$D$22*SIN(RADIANS(H25))</f>
-        <v>97.347463868399842</v>
-      </c>
-      <c r="L25" s="14">
+      <c r="T25" s="8">
+        <f>AC25-H4</f>
+        <v>-4.3041489472911785</v>
+      </c>
+      <c r="U25" s="9">
         <f t="shared" si="0"/>
-        <v>184.68132734448011</v>
-      </c>
-      <c r="M25" s="14">
+        <v>209.52782734134087</v>
+      </c>
+      <c r="V25" s="9">
         <f t="shared" si="1"/>
-        <v>171.12502270416508</v>
-      </c>
-      <c r="N25" s="15">
+        <v>98.088184662310283</v>
+      </c>
+      <c r="W25" s="9">
         <f t="shared" si="2"/>
-        <v>65.697995437448327</v>
-      </c>
-      <c r="O25" s="14">
+        <v>146.3333828843476</v>
+      </c>
+      <c r="X25" s="9">
         <f t="shared" si="3"/>
-        <v>0.38448311308417726</v>
-      </c>
-      <c r="P25" s="14">
+        <v>110.75210012740075</v>
+      </c>
+      <c r="Y25" s="10">
         <f t="shared" si="4"/>
-        <v>263.29890067641236</v>
-      </c>
-      <c r="Q25" s="14">
+        <v>56.86802543934683</v>
+      </c>
+      <c r="Z25" s="9">
         <f t="shared" si="5"/>
-        <v>31.230045047428305</v>
-      </c>
-      <c r="R25" s="13">
-        <f>-DEGREES(ATAN((J25-P25)/(K25-Q25)))</f>
-        <v>9.7282459730292103</v>
+        <v>0.5501152878514004</v>
+      </c>
+      <c r="AA25" s="9">
+        <f t="shared" si="6"/>
+        <v>204.49325752884434</v>
+      </c>
+      <c r="AB25" s="9">
+        <f t="shared" si="7"/>
+        <v>31.195336712749189</v>
+      </c>
+      <c r="AC25" s="8">
+        <f t="shared" si="8"/>
+        <v>-4.3041489472911785</v>
       </c>
     </row>
-    <row r="26" spans="3:18" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="26" spans="3:29" ht="15.75" x14ac:dyDescent="0.3">
       <c r="C26" s="2" t="s">
         <v>26</v>
       </c>
@@ -3680,51 +3746,51 @@
       <c r="F26" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="H26" s="11">
+      <c r="S26" s="6">
         <v>-2</v>
       </c>
-      <c r="I26" s="13">
-        <f>R26-5</f>
-        <v>4.787301670100236</v>
-      </c>
-      <c r="J26" s="14">
-        <f>$D$5+$D$22*COS(RADIANS(H26))</f>
-        <v>251.89425525839013</v>
-      </c>
-      <c r="K26" s="14">
-        <f>$D$6+$D$22*SIN(RADIANS(H26))</f>
-        <v>94.695735725001072</v>
-      </c>
-      <c r="L26" s="14">
+      <c r="T26" s="8">
+        <f>AC26-H4</f>
+        <v>-4.258150890240632</v>
+      </c>
+      <c r="U26" s="9">
         <f t="shared" si="0"/>
-        <v>183.66592828240016</v>
-      </c>
-      <c r="M26" s="14">
+        <v>209.47777994442043</v>
+      </c>
+      <c r="V26" s="9">
         <f t="shared" si="1"/>
-        <v>171.05288335032134</v>
-      </c>
-      <c r="N26" s="15">
+        <v>96.176951682092607</v>
+      </c>
+      <c r="W26" s="9">
         <f t="shared" si="2"/>
-        <v>65.885590970570746</v>
-      </c>
-      <c r="O26" s="14">
+        <v>145.40936845083186</v>
+      </c>
+      <c r="X26" s="9">
         <f t="shared" si="3"/>
-        <v>-0.44072276433740876</v>
-      </c>
-      <c r="P26" s="14">
+        <v>110.52893213045891</v>
+      </c>
+      <c r="Y26" s="10">
         <f t="shared" si="4"/>
-        <v>263.29760500302513</v>
-      </c>
-      <c r="Q26" s="14">
+        <v>57.300568601894412</v>
+      </c>
+      <c r="Z26" s="9">
         <f t="shared" si="5"/>
-        <v>28.590035406484475</v>
-      </c>
-      <c r="R26" s="13">
-        <f>-DEGREES(ATAN((J26-P26)/(K26-Q26)))</f>
-        <v>9.787301670100236</v>
+        <v>-0.33131520089371436</v>
+      </c>
+      <c r="AA26" s="9">
+        <f t="shared" si="6"/>
+        <v>204.49691450055795</v>
+      </c>
+      <c r="AB26" s="9">
+        <f t="shared" si="7"/>
+        <v>29.280083448743021</v>
+      </c>
+      <c r="AC26" s="8">
+        <f t="shared" si="8"/>
+        <v>-4.258150890240632</v>
       </c>
     </row>
-    <row r="27" spans="3:18" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="27" spans="3:29" ht="15.75" x14ac:dyDescent="0.3">
       <c r="C27" s="2" t="s">
         <v>29</v>
       </c>
@@ -3739,57 +3805,57 @@
         <v>49</v>
       </c>
       <c r="G27" s="3"/>
-      <c r="H27" s="11">
+      <c r="S27" s="6">
         <v>-3</v>
       </c>
-      <c r="I27" s="13">
-        <f>R27-5</f>
-        <v>4.8535715108811956</v>
-      </c>
-      <c r="J27" s="14">
-        <f>$D$5+$D$22*COS(RADIANS(H27))</f>
-        <v>251.77854885161986</v>
-      </c>
-      <c r="K27" s="14">
-        <f>$D$6+$D$22*SIN(RADIANS(H27))</f>
-        <v>92.045623311884015</v>
-      </c>
-      <c r="L27" s="14">
+      <c r="T27" s="8">
+        <f>AC27-H4</f>
+        <v>-4.2088149983734144</v>
+      </c>
+      <c r="U27" s="9">
         <f t="shared" si="0"/>
-        <v>182.64043697310998</v>
-      </c>
-      <c r="M27" s="14">
+        <v>209.39438455519388</v>
+      </c>
+      <c r="V27" s="9">
         <f t="shared" si="1"/>
-        <v>170.98494247175975</v>
-      </c>
-      <c r="N27" s="15">
+        <v>94.266883239427273</v>
+      </c>
+      <c r="W27" s="9">
         <f t="shared" si="2"/>
-        <v>66.061709393028892</v>
-      </c>
-      <c r="O27" s="14">
+        <v>144.47539249203504</v>
+      </c>
+      <c r="X27" s="9">
         <f t="shared" si="3"/>
-        <v>-1.2650412166590148</v>
-      </c>
-      <c r="P27" s="14">
+        <v>110.30646287216263</v>
+      </c>
+      <c r="Y27" s="10">
         <f t="shared" si="4"/>
-        <v>263.25835058390402</v>
-      </c>
-      <c r="Q27" s="14">
+        <v>57.727673161424136</v>
+      </c>
+      <c r="Z27" s="9">
         <f t="shared" si="5"/>
-        <v>25.953156629307763</v>
-      </c>
-      <c r="R27" s="13">
-        <f>-DEGREES(ATAN((J27-P27)/(K27-Q27)))</f>
-        <v>9.8535715108811956</v>
+        <v>-1.2124002907446598</v>
+      </c>
+      <c r="AA27" s="9">
+        <f t="shared" si="6"/>
+        <v>204.47112408809895</v>
+      </c>
+      <c r="AB27" s="9">
+        <f t="shared" si="7"/>
+        <v>27.365750914382552</v>
+      </c>
+      <c r="AC27" s="8">
+        <f t="shared" si="8"/>
+        <v>-4.2088149983734144</v>
       </c>
     </row>
-    <row r="28" spans="3:18" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="28" spans="3:29" ht="15.75" x14ac:dyDescent="0.3">
       <c r="C28" s="2" t="s">
         <v>50</v>
       </c>
       <c r="D28" s="2">
         <f>D5+D22*COS(RADIANS(D16))</f>
-        <v>249.6778199002018</v>
+        <v>209.54451150103324</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>21</v>
@@ -3797,57 +3863,57 @@
       <c r="F28" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="H28" s="11">
+      <c r="S28" s="6">
         <v>-4</v>
       </c>
-      <c r="I28" s="13">
-        <f>R28-5</f>
-        <v>4.9271524933254724</v>
-      </c>
-      <c r="J28" s="14">
-        <f>$D$5+$D$22*COS(RADIANS(H28))</f>
-        <v>251.61660922855759</v>
-      </c>
-      <c r="K28" s="14">
-        <f>$D$6+$D$22*SIN(RADIANS(H28))</f>
-        <v>89.39793387896195</v>
-      </c>
-      <c r="L28" s="14">
+      <c r="T28" s="8">
+        <f>AC28-H4</f>
+        <v>-4.1561244320006185</v>
+      </c>
+      <c r="U28" s="9">
         <f t="shared" si="0"/>
-        <v>181.60499748684498</v>
-      </c>
-      <c r="M28" s="14">
+        <v>209.2776665767046</v>
+      </c>
+      <c r="V28" s="9">
         <f t="shared" si="1"/>
-        <v>170.92143930866746</v>
-      </c>
-      <c r="N28" s="15">
+        <v>92.358561159665143</v>
+      </c>
+      <c r="W28" s="9">
         <f t="shared" si="2"/>
-        <v>66.225837742179593</v>
-      </c>
-      <c r="O28" s="14">
+        <v>143.53154784026162</v>
+      </c>
+      <c r="X28" s="9">
         <f t="shared" si="3"/>
-        <v>-2.0883747438679521</v>
-      </c>
-      <c r="P28" s="14">
+        <v>110.08487576748935</v>
+      </c>
+      <c r="Y28" s="10">
         <f t="shared" si="4"/>
-        <v>263.18127942661272</v>
-      </c>
-      <c r="Q28" s="14">
+        <v>58.14911974618736</v>
+      </c>
+      <c r="Z28" s="9">
         <f t="shared" si="5"/>
-        <v>23.320264404242891</v>
-      </c>
-      <c r="R28" s="13">
-        <f>-DEGREES(ATAN((J28-P28)/(K28-Q28)))</f>
-        <v>9.9271524933254724</v>
+        <v>-2.093076317312963</v>
+      </c>
+      <c r="AA28" s="9">
+        <f t="shared" si="6"/>
+        <v>204.41593206083689</v>
+      </c>
+      <c r="AB28" s="9">
+        <f t="shared" si="7"/>
+        <v>25.452929576836333</v>
+      </c>
+      <c r="AC28" s="8">
+        <f t="shared" si="8"/>
+        <v>-4.1561244320006185</v>
       </c>
     </row>
-    <row r="29" spans="3:18" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="29" spans="3:29" ht="15.75" x14ac:dyDescent="0.3">
       <c r="C29" s="2" t="s">
         <v>52</v>
       </c>
       <c r="D29" s="2">
         <f>D6+D22*SIN(RADIANS(D16))</f>
-        <v>126.39223806202797</v>
+        <v>100</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>21</v>
@@ -3855,57 +3921,57 @@
       <c r="F29" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="H29" s="11">
+      <c r="S29" s="6">
         <v>-5</v>
       </c>
-      <c r="I29" s="13">
-        <f>R29-5</f>
-        <v>5.0081525952775916</v>
-      </c>
-      <c r="J29" s="14">
-        <f>$D$5+$D$22*COS(RADIANS(H29))</f>
-        <v>251.40848571758124</v>
-      </c>
-      <c r="K29" s="14">
-        <f>$D$6+$D$22*SIN(RADIANS(H29))</f>
-        <v>86.753473938084866</v>
-      </c>
-      <c r="L29" s="14">
+      <c r="T29" s="8">
+        <f>AC29-H4</f>
+        <v>-4.1000578137126542</v>
+      </c>
+      <c r="U29" s="9">
         <f t="shared" si="0"/>
-        <v>180.55975681207352</v>
-      </c>
-      <c r="M29" s="14">
+        <v>209.12766156237956</v>
+      </c>
+      <c r="V29" s="9">
         <f t="shared" si="1"/>
-        <v>170.86261875134875</v>
-      </c>
-      <c r="N29" s="15">
+        <v>90.452566736198065</v>
+      </c>
+      <c r="W29" s="9">
         <f t="shared" si="2"/>
-        <v>66.377447325362255</v>
-      </c>
-      <c r="O29" s="14">
+        <v>142.57792888649672</v>
+      </c>
+      <c r="X29" s="9">
         <f t="shared" si="3"/>
-        <v>-2.9106228007657569</v>
-      </c>
-      <c r="P29" s="14">
+        <v>109.86435996872575</v>
+      </c>
+      <c r="Y29" s="10">
         <f t="shared" si="4"/>
-        <v>263.06655954997046</v>
-      </c>
-      <c r="Q29" s="14">
+        <v>58.56468567884788</v>
+      </c>
+      <c r="Z29" s="9">
         <f t="shared" si="5"/>
-        <v>20.692219677220585</v>
-      </c>
-      <c r="R29" s="13">
-        <f>-DEGREES(ATAN((J29-P29)/(K29-Q29)))</f>
-        <v>10.008152595277592</v>
+        <v>-2.9732789552005254</v>
+      </c>
+      <c r="AA29" s="9">
+        <f t="shared" si="6"/>
+        <v>204.3313996748129</v>
+      </c>
+      <c r="AB29" s="9">
+        <f t="shared" si="7"/>
+        <v>23.54220975085628</v>
+      </c>
+      <c r="AC29" s="8">
+        <f t="shared" si="8"/>
+        <v>-4.1000578137126542</v>
       </c>
     </row>
-    <row r="30" spans="3:18" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="30" spans="3:29" ht="15.75" x14ac:dyDescent="0.3">
       <c r="C30" s="4" t="s">
         <v>54</v>
       </c>
       <c r="D30" s="4">
         <f>SQRT((D28-D7)^2 + (D29-D8)^2)</f>
-        <v>195.14616605173669</v>
+        <v>147.24734449232466</v>
       </c>
       <c r="E30" s="4" t="s">
         <v>21</v>
@@ -3913,57 +3979,57 @@
       <c r="F30" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="H30" s="11">
+      <c r="S30" s="6">
         <v>-6</v>
       </c>
-      <c r="I30" s="13">
-        <f>R30-5</f>
-        <v>5.096691346211756</v>
-      </c>
-      <c r="J30" s="14">
-        <f>$D$5+$D$22*COS(RADIANS(H30))</f>
-        <v>251.15424171512836</v>
-      </c>
-      <c r="K30" s="14">
-        <f>$D$6+$D$22*SIN(RADIANS(H30))</f>
-        <v>84.113049017368212</v>
-      </c>
-      <c r="L30" s="14">
+      <c r="T30" s="8">
+        <f>AC30-H4</f>
+        <v>-4.0405891570269974</v>
+      </c>
+      <c r="U30" s="9">
         <f t="shared" si="0"/>
-        <v>179.50486492303401</v>
-      </c>
-      <c r="M30" s="14">
+        <v>208.94441520519916</v>
+      </c>
+      <c r="V30" s="9">
         <f t="shared" si="1"/>
-        <v>170.80873144393499</v>
-      </c>
-      <c r="N30" s="15">
+        <v>88.549480553391206</v>
+      </c>
+      <c r="W30" s="9">
         <f t="shared" si="2"/>
-        <v>66.515992531974504</v>
-      </c>
-      <c r="O30" s="14">
+        <v>141.61463160875266</v>
+      </c>
+      <c r="X30" s="9">
         <f t="shared" si="3"/>
-        <v>-3.731681518826246</v>
-      </c>
-      <c r="P30" s="14">
+        <v>109.64511058249774</v>
+      </c>
+      <c r="Y30" s="10">
         <f t="shared" si="4"/>
-        <v>262.91438556280644</v>
-      </c>
-      <c r="Q30" s="14">
+        <v>58.974144549555291</v>
+      </c>
+      <c r="Z30" s="9">
         <f t="shared" si="5"/>
-        <v>18.069888760745762</v>
-      </c>
-      <c r="R30" s="13">
-        <f>-DEGREES(ATAN((J30-P30)/(K30-Q30)))</f>
-        <v>10.096691346211756</v>
+        <v>-3.852943082745548</v>
+      </c>
+      <c r="AA30" s="9">
+        <f t="shared" si="6"/>
+        <v>204.21760374469244</v>
+      </c>
+      <c r="AB30" s="9">
+        <f t="shared" si="7"/>
+        <v>21.634181455077218</v>
+      </c>
+      <c r="AC30" s="8">
+        <f t="shared" si="8"/>
+        <v>-4.0405891570269974</v>
       </c>
     </row>
-    <row r="31" spans="3:18" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="31" spans="3:29" ht="15.75" x14ac:dyDescent="0.3">
       <c r="C31" s="4" t="s">
         <v>56</v>
       </c>
       <c r="D31" s="5">
         <f>(D23^2 - D27^2 + D30^2)/(2*D30)</f>
-        <v>172.13258011659028</v>
+        <v>110.97578897847251</v>
       </c>
       <c r="E31" s="4" t="s">
         <v>21</v>
@@ -3971,57 +4037,57 @@
       <c r="F31" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="H31" s="11">
+      <c r="S31" s="6">
         <v>-7</v>
       </c>
-      <c r="I31" s="13">
-        <f>R31-5</f>
-        <v>5.1929004565316337</v>
-      </c>
-      <c r="J31" s="14">
-        <f>$D$5+$D$22*COS(RADIANS(H31))</f>
-        <v>250.85395466638505</v>
-      </c>
-      <c r="K31" s="14">
-        <f>$D$6+$D$22*SIN(RADIANS(H31))</f>
-        <v>81.477463415821234</v>
-      </c>
-      <c r="L31" s="14">
+      <c r="T31" s="8">
+        <f>AC31-H4</f>
+        <v>-3.9776877803165664</v>
+      </c>
+      <c r="U31" s="9">
         <f t="shared" si="0"/>
-        <v>178.44047485049566</v>
-      </c>
-      <c r="M31" s="14">
+        <v>208.72798332377909</v>
+      </c>
+      <c r="V31" s="9">
         <f t="shared" si="1"/>
-        <v>170.76003388785281</v>
-      </c>
-      <c r="N31" s="15">
+        <v>86.649882309731453</v>
+      </c>
+      <c r="W31" s="9">
         <f t="shared" si="2"/>
-        <v>66.640909557263342</v>
-      </c>
-      <c r="O31" s="14">
+        <v>140.64175360224135</v>
+      </c>
+      <c r="X31" s="9">
         <f t="shared" si="3"/>
-        <v>-4.5514434053736812</v>
-      </c>
-      <c r="P31" s="14">
+        <v>109.4273288975225</v>
+      </c>
+      <c r="Y31" s="10">
         <f t="shared" si="4"/>
-        <v>262.72497929494324</v>
-      </c>
-      <c r="Q31" s="14">
+        <v>59.377265770271343</v>
+      </c>
+      <c r="Z31" s="9">
         <f t="shared" si="5"/>
-        <v>15.454143488176264</v>
-      </c>
-      <c r="R31" s="13">
-        <f>-DEGREES(ATAN((J31-P31)/(K31-Q31)))</f>
-        <v>10.192900456531634</v>
+        <v>-4.7320026425792179</v>
+      </c>
+      <c r="AA31" s="9">
+        <f t="shared" si="6"/>
+        <v>204.07463672983801</v>
+      </c>
+      <c r="AB31" s="9">
+        <f t="shared" si="7"/>
+        <v>19.729434272702754</v>
+      </c>
+      <c r="AC31" s="8">
+        <f t="shared" si="8"/>
+        <v>-3.9776877803165664</v>
       </c>
     </row>
-    <row r="32" spans="3:18" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="32" spans="3:29" ht="15.75" x14ac:dyDescent="0.3">
       <c r="C32" s="4" t="s">
         <v>58</v>
       </c>
       <c r="D32" s="5">
         <f>SQRT(D23^2 - D31^2)</f>
-        <v>63.010910661611803</v>
+        <v>56.430260150078524</v>
       </c>
       <c r="E32" s="4" t="s">
         <v>21</v>
@@ -4029,57 +4095,57 @@
       <c r="F32" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="H32" s="11">
+      <c r="S32" s="6">
         <v>-8</v>
       </c>
-      <c r="I32" s="13">
-        <f>R32-5</f>
-        <v>5.2969245106614267</v>
-      </c>
-      <c r="J32" s="14">
-        <f>$D$5+$D$22*COS(RADIANS(H32))</f>
-        <v>250.50771604169532</v>
-      </c>
-      <c r="K32" s="14">
-        <f>$D$6+$D$22*SIN(RADIANS(H32))</f>
-        <v>78.847519958349636</v>
-      </c>
-      <c r="L32" s="14">
+      <c r="T32" s="8">
+        <f>AC32-H4</f>
+        <v>-3.9113182053348545</v>
+      </c>
+      <c r="U32" s="9">
         <f t="shared" si="0"/>
-        <v>177.36674275589763</v>
-      </c>
-      <c r="M32" s="14">
+        <v>208.47843184536691</v>
+      </c>
+      <c r="V32" s="9">
         <f t="shared" si="1"/>
-        <v>170.71678854468647</v>
-      </c>
-      <c r="N32" s="15">
+        <v>84.754350641245651</v>
+      </c>
+      <c r="W32" s="9">
         <f t="shared" si="2"/>
-        <v>66.751615029067281</v>
-      </c>
-      <c r="O32" s="14">
+        <v>139.65939411149208</v>
+      </c>
+      <c r="X32" s="9">
         <f t="shared" si="3"/>
-        <v>-5.3697970176106153</v>
-      </c>
-      <c r="P32" s="14">
+        <v>109.21122262365213</v>
+      </c>
+      <c r="Y32" s="10">
         <f t="shared" si="4"/>
-        <v>262.49859048638177</v>
-      </c>
-      <c r="Q32" s="14">
+        <v>59.773814108245531</v>
+      </c>
+      <c r="Z32" s="9">
         <f t="shared" si="5"/>
-        <v>12.845861418190424</v>
-      </c>
-      <c r="R32" s="13">
-        <f>-DEGREES(ATAN((J32-P32)/(K32-Q32)))</f>
-        <v>10.296924510661427</v>
+        <v>-5.6103904973618848</v>
+      </c>
+      <c r="AA32" s="9">
+        <f t="shared" si="6"/>
+        <v>203.90260683527981</v>
+      </c>
+      <c r="AB32" s="9">
+        <f t="shared" si="7"/>
+        <v>17.828557216908401</v>
+      </c>
+      <c r="AC32" s="8">
+        <f t="shared" si="8"/>
+        <v>-3.9113182053348545</v>
       </c>
     </row>
-    <row r="33" spans="3:18" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="33" spans="3:29" ht="15.75" x14ac:dyDescent="0.3">
       <c r="C33" s="4" t="s">
         <v>60</v>
       </c>
       <c r="D33" s="5">
         <f>D7 + D31*(D28-D7)/D30</f>
-        <v>229.66771584042576</v>
+        <v>177.63370892170718</v>
       </c>
       <c r="E33" s="4" t="s">
         <v>21</v>
@@ -4087,57 +4153,57 @@
       <c r="F33" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="H33" s="11">
+      <c r="S33" s="6">
         <v>-9</v>
       </c>
-      <c r="I33" s="13">
-        <f>R33-5</f>
-        <v>5.4089217309654174</v>
-      </c>
-      <c r="J33" s="14">
-        <f>$D$5+$D$22*COS(RADIANS(H33))</f>
-        <v>250.11563130869825</v>
-      </c>
-      <c r="K33" s="14">
-        <f>$D$6+$D$22*SIN(RADIANS(H33))</f>
-        <v>76.224019751207393</v>
-      </c>
-      <c r="L33" s="14">
+      <c r="T33" s="8">
+        <f>AC33-H4</f>
+        <v>-3.8414400395590254</v>
+      </c>
+      <c r="U33" s="9">
         <f t="shared" si="0"/>
-        <v>176.28382800902915</v>
-      </c>
-      <c r="M33" s="14">
+        <v>208.19583678576049</v>
+      </c>
+      <c r="V33" s="9">
         <f t="shared" si="1"/>
-        <v>170.67926393802497</v>
-      </c>
-      <c r="N33" s="15">
+        <v>82.863462945242446</v>
+      </c>
+      <c r="W33" s="9">
         <f t="shared" si="2"/>
-        <v>66.84750452764861</v>
-      </c>
-      <c r="O33" s="14">
+        <v>138.66765406454513</v>
+      </c>
+      <c r="X33" s="9">
         <f t="shared" si="3"/>
-        <v>-6.1866266086976003</v>
-      </c>
-      <c r="P33" s="14">
+        <v>108.9970061428093</v>
+      </c>
+      <c r="Y33" s="10">
         <f t="shared" si="4"/>
-        <v>262.23549754138867</v>
-      </c>
-      <c r="Q33" s="14">
+        <v>60.16354919637299</v>
+      </c>
+      <c r="Z33" s="9">
         <f t="shared" si="5"/>
-        <v>10.245926095042364</v>
-      </c>
-      <c r="R33" s="13">
-        <f>-DEGREES(ATAN((J33-P33)/(K33-Q33)))</f>
-        <v>10.408921730965417</v>
+        <v>-6.4880382800219376</v>
+      </c>
+      <c r="AA33" s="9">
+        <f t="shared" si="6"/>
+        <v>203.70163812847451</v>
+      </c>
+      <c r="AB33" s="9">
+        <f t="shared" si="7"/>
+        <v>15.932138601338643</v>
+      </c>
+      <c r="AC33" s="8">
+        <f t="shared" si="8"/>
+        <v>-3.8414400395590254</v>
       </c>
     </row>
-    <row r="34" spans="3:18" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="34" spans="3:29" ht="15.75" x14ac:dyDescent="0.3">
       <c r="C34" s="4" t="s">
         <v>62</v>
       </c>
       <c r="D34" s="5">
         <f>D8 + D31*(D29-D8)/D30</f>
-        <v>115.02470213240353</v>
+        <v>82.756844310343411</v>
       </c>
       <c r="E34" s="4" t="s">
         <v>21</v>
@@ -4145,51 +4211,51 @@
       <c r="F34" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="H34" s="11">
+      <c r="S34" s="6">
         <v>-10</v>
       </c>
-      <c r="I34" s="13">
-        <f>R34-5</f>
-        <v>5.529064820462489</v>
-      </c>
-      <c r="J34" s="14">
-        <f>$D$5+$D$22*COS(RADIANS(H34))</f>
-        <v>249.6778199002018</v>
-      </c>
-      <c r="K34" s="14">
-        <f>$D$6+$D$22*SIN(RADIANS(H34))</f>
-        <v>73.607761937972029</v>
-      </c>
-      <c r="L34" s="14">
+      <c r="T34" s="8">
+        <f>AC34-H4</f>
+        <v>-3.7680078414639691</v>
+      </c>
+      <c r="U34" s="9">
         <f t="shared" si="0"/>
-        <v>175.19189326942089</v>
-      </c>
-      <c r="M34" s="14">
+        <v>207.88028422615253</v>
+      </c>
+      <c r="V34" s="9">
         <f t="shared" si="1"/>
-        <v>170.6477347538337</v>
-      </c>
-      <c r="N34" s="15">
+        <v>80.977795204431487</v>
+      </c>
+      <c r="W34" s="9">
         <f t="shared" si="2"/>
-        <v>66.927950987500054</v>
-      </c>
-      <c r="O34" s="14">
+        <v>137.66663610935845</v>
+      </c>
+      <c r="X34" s="9">
         <f t="shared" si="3"/>
-        <v>-7.0018117427115403</v>
-      </c>
-      <c r="P34" s="14">
+        <v>108.78490077244794</v>
+      </c>
+      <c r="Y34" s="10">
         <f t="shared" si="4"/>
-        <v>261.93600835502247</v>
-      </c>
-      <c r="Q34" s="14">
+        <v>60.546225017986515</v>
+      </c>
+      <c r="Z34" s="9">
         <f t="shared" si="5"/>
-        <v>7.6552273710117333</v>
-      </c>
-      <c r="R34" s="13">
-        <f>-DEGREES(ATAN((J34-P34)/(K34-Q34)))</f>
-        <v>10.529064820462489</v>
+        <v>-7.3648762377676062</v>
+      </c>
+      <c r="AA34" s="9">
+        <f t="shared" si="6"/>
+        <v>203.47187067286291</v>
+      </c>
+      <c r="AB34" s="9">
+        <f t="shared" si="7"/>
+        <v>14.040765916128201</v>
+      </c>
+      <c r="AC34" s="8">
+        <f t="shared" si="8"/>
+        <v>-3.7680078414639691</v>
       </c>
     </row>
-    <row r="35" spans="3:18" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="35" spans="3:29" ht="15.75" x14ac:dyDescent="0.3">
       <c r="C35" s="4" t="s">
         <v>64</v>
       </c>
@@ -4202,57 +4268,57 @@
       <c r="F35" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="H35" s="11">
+      <c r="S35" s="6">
         <v>-11</v>
       </c>
-      <c r="I35" s="13">
-        <f>R35-5</f>
-        <v>5.6575418933853232</v>
-      </c>
-      <c r="J35" s="14">
-        <f>$D$5+$D$22*COS(RADIANS(H35))</f>
-        <v>249.19441517780214</v>
-      </c>
-      <c r="K35" s="14">
-        <f>$D$6+$D$22*SIN(RADIANS(H35))</f>
-        <v>70.999543456117706</v>
-      </c>
-      <c r="L35" s="14">
+      <c r="T35" s="8">
+        <f>AC35-H4</f>
+        <v>-3.6909709677256304</v>
+      </c>
+      <c r="U35" s="9">
         <f t="shared" si="0"/>
-        <v>174.09110457162527</v>
-      </c>
-      <c r="M35" s="14">
+        <v>207.53187028690948</v>
+      </c>
+      <c r="V35" s="9">
         <f t="shared" si="1"/>
-        <v>170.62248193883681</v>
-      </c>
-      <c r="N35" s="15">
+        <v>79.097921811473498</v>
+      </c>
+      <c r="W35" s="9">
         <f t="shared" si="2"/>
-        <v>66.992302968559741</v>
-      </c>
-      <c r="O35" s="14">
+        <v>136.65644465257637</v>
+      </c>
+      <c r="X35" s="9">
         <f t="shared" si="3"/>
-        <v>-7.815226874873666</v>
-      </c>
-      <c r="P35" s="14">
+        <v>108.57513504220677</v>
+      </c>
+      <c r="Y35" s="10">
         <f t="shared" si="4"/>
-        <v>261.60046122060356</v>
-      </c>
-      <c r="Q35" s="14">
+        <v>60.921589363431444</v>
+      </c>
+      <c r="Z35" s="9">
         <f t="shared" si="5"/>
-        <v>5.0746617984015359</v>
-      </c>
-      <c r="R35" s="13">
-        <f>-DEGREES(ATAN((J35-P35)/(K35-Q35)))</f>
-        <v>10.657541893385323</v>
+        <v>-8.2408330690834983</v>
+      </c>
+      <c r="AA35" s="9">
+        <f t="shared" si="6"/>
+        <v>203.21346067937091</v>
+      </c>
+      <c r="AB35" s="9">
+        <f t="shared" si="7"/>
+        <v>12.155025709933952</v>
+      </c>
+      <c r="AC35" s="8">
+        <f t="shared" si="8"/>
+        <v>-3.6909709677256304</v>
       </c>
     </row>
-    <row r="36" spans="3:18" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="36" spans="3:29" ht="15.75" x14ac:dyDescent="0.3">
       <c r="C36" s="2" t="s">
         <v>67</v>
       </c>
       <c r="D36" s="1">
         <f>D33 - D35*D32*(D29-D8)/D30</f>
-        <v>260.79188714179276</v>
+        <v>204.46012283174818</v>
       </c>
       <c r="E36" s="2" t="s">
         <v>21</v>
@@ -4260,57 +4326,57 @@
       <c r="F36" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="H36" s="11">
+      <c r="S36" s="6">
         <v>-12</v>
       </c>
-      <c r="I36" s="13">
-        <f>R36-5</f>
-        <v>5.7945575038849313</v>
-      </c>
-      <c r="J36" s="14">
-        <f>$D$5+$D$22*COS(RADIANS(H36))</f>
-        <v>248.66556439126057</v>
-      </c>
-      <c r="K36" s="14">
-        <f>$D$6+$D$22*SIN(RADIANS(H36))</f>
-        <v>68.400158794260378</v>
-      </c>
-      <c r="L36" s="14">
+      <c r="T36" s="8">
+        <f>AC36-H4</f>
+        <v>-3.6102734012226483</v>
+      </c>
+      <c r="U36" s="9">
         <f t="shared" si="0"/>
-        <v>172.98163141457212</v>
-      </c>
-      <c r="M36" s="14">
+        <v>207.15070109829242</v>
+      </c>
+      <c r="V36" s="9">
         <f t="shared" si="1"/>
-        <v>170.60379279633375</v>
-      </c>
-      <c r="N36" s="15">
+        <v>77.224415394014699</v>
+      </c>
+      <c r="W36" s="9">
         <f t="shared" si="2"/>
-        <v>67.039882782606441</v>
-      </c>
-      <c r="O36" s="14">
+        <v>135.63718590082055</v>
+      </c>
+      <c r="X36" s="9">
         <f t="shared" si="3"/>
-        <v>-8.6267408929373879</v>
-      </c>
-      <c r="P36" s="14">
+        <v>108.36794498445839</v>
+      </c>
+      <c r="Y36" s="10">
         <f t="shared" si="4"/>
-        <v>261.22922582774936</v>
-      </c>
-      <c r="Q36" s="14">
+        <v>61.289383255547605</v>
+      </c>
+      <c r="Z36" s="9">
         <f t="shared" si="5"/>
-        <v>2.5051330995292034</v>
-      </c>
-      <c r="R36" s="13">
-        <f>-DEGREES(ATAN((J36-P36)/(K36-Q36)))</f>
-        <v>10.794557503884931</v>
+        <v>-9.1158357528572029</v>
+      </c>
+      <c r="AA36" s="9">
+        <f t="shared" si="6"/>
+        <v>202.92658067714413</v>
+      </c>
+      <c r="AB36" s="9">
+        <f t="shared" si="7"/>
+        <v>10.275503478527696</v>
+      </c>
+      <c r="AC36" s="8">
+        <f t="shared" si="8"/>
+        <v>-3.6102734012226483</v>
       </c>
     </row>
-    <row r="37" spans="3:18" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="37" spans="3:29" ht="15.75" x14ac:dyDescent="0.3">
       <c r="C37" s="2" t="s">
         <v>68</v>
       </c>
       <c r="D37" s="1">
         <f>D34 + D35*D32*(D28-D7)/D30</f>
-        <v>60.237287307383838</v>
+        <v>33.110920234617922</v>
       </c>
       <c r="E37" s="2" t="s">
         <v>21</v>
@@ -4318,57 +4384,57 @@
       <c r="F37" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="H37" s="11">
+      <c r="S37" s="6">
         <v>-13</v>
       </c>
-      <c r="I37" s="13">
-        <f>R37-5</f>
-        <v>5.9403337846479189</v>
-      </c>
-      <c r="J37" s="14">
-        <f>$D$5+$D$22*COS(RADIANS(H37))</f>
-        <v>248.09142863364977</v>
-      </c>
-      <c r="K37" s="14">
-        <f>$D$6+$D$22*SIN(RADIANS(H37))</f>
-        <v>65.810399750148861</v>
-      </c>
-      <c r="L37" s="14">
+      <c r="T37" s="8">
+        <f>AC37-H4</f>
+        <v>-3.5258535585610882</v>
+      </c>
+      <c r="U37" s="9">
         <f t="shared" si="0"/>
-        <v>171.86364685519399</v>
-      </c>
-      <c r="M37" s="14">
+        <v>206.73689276812871</v>
+      </c>
+      <c r="V37" s="9">
         <f t="shared" si="1"/>
-        <v>170.59196107880891</v>
-      </c>
-      <c r="N37" s="15">
+        <v>75.357846640258927</v>
+      </c>
+      <c r="W37" s="9">
         <f t="shared" si="2"/>
-        <v>67.069984458669282</v>
-      </c>
-      <c r="O37" s="14">
+        <v>134.60896790467345</v>
+      </c>
+      <c r="X37" s="9">
         <f t="shared" si="3"/>
-        <v>-9.4362166150407791</v>
-      </c>
-      <c r="P37" s="14">
+        <v>108.16357443949472</v>
+      </c>
+      <c r="Y37" s="10">
         <f t="shared" si="4"/>
-        <v>260.82270436189685</v>
-      </c>
-      <c r="Q37" s="14">
+        <v>61.649340340930515</v>
+      </c>
+      <c r="Z37" s="9">
         <f t="shared" si="5"/>
-        <v>-5.2447275555593365E-2</v>
-      </c>
-      <c r="R37" s="13">
-        <f>-DEGREES(ATAN((J37-P37)/(K37-Q37)))</f>
-        <v>10.940333784647919</v>
+        <v>-9.9898093687065366</v>
+      </c>
+      <c r="AA37" s="9">
+        <f t="shared" si="6"/>
+        <v>202.61141970497042</v>
+      </c>
+      <c r="AB37" s="9">
+        <f t="shared" si="7"/>
+        <v>8.4027835605697732</v>
+      </c>
+      <c r="AC37" s="8">
+        <f t="shared" si="8"/>
+        <v>-3.5258535585610882</v>
       </c>
     </row>
-    <row r="38" spans="3:18" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="38" spans="3:29" ht="15.75" x14ac:dyDescent="0.3">
       <c r="C38" s="2" t="s">
         <v>28</v>
       </c>
       <c r="D38" s="1">
         <f>DEGREES(ATAN2(D36-D7, D37-D8))</f>
-        <v>9.4947903177358484</v>
+        <v>1.4318280404579051</v>
       </c>
       <c r="E38" s="2" t="s">
         <v>1</v>
@@ -4376,147 +4442,147 @@
       <c r="F38" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="H38" s="11">
+      <c r="S38" s="6">
         <v>-14</v>
       </c>
-      <c r="I38" s="13">
-        <f>R38-5</f>
-        <v>6.0951117088974627</v>
-      </c>
-      <c r="J38" s="14">
-        <f>$D$5+$D$22*COS(RADIANS(H38))</f>
-        <v>247.47218279228326</v>
-      </c>
-      <c r="K38" s="14">
-        <f>$D$6+$D$22*SIN(RADIANS(H38))</f>
-        <v>63.231055189475533</v>
-      </c>
-      <c r="L38" s="14">
+      <c r="T38" s="8">
+        <f>AC38-H4</f>
+        <v>-3.4376440756897959</v>
+      </c>
+      <c r="U38" s="9">
         <f t="shared" si="0"/>
-        <v>170.73732760652518</v>
-      </c>
-      <c r="M38" s="14">
+        <v>206.29057134644427</v>
+      </c>
+      <c r="V38" s="9">
         <f t="shared" si="1"/>
-        <v>170.58728707661837</v>
-      </c>
-      <c r="N38" s="15">
+        <v>73.498784125130442</v>
+      </c>
+      <c r="W38" s="9">
         <f t="shared" si="2"/>
-        <v>67.081871529045642</v>
-      </c>
-      <c r="O38" s="14">
+        <v>133.57190060553916</v>
+      </c>
+      <c r="X38" s="9">
         <f t="shared" si="3"/>
-        <v>-10.243510238649691</v>
-      </c>
-      <c r="P38" s="14">
+        <v>107.96227537612799</v>
+      </c>
+      <c r="Y38" s="10">
         <f t="shared" si="4"/>
-        <v>260.38133271773859</v>
-      </c>
-      <c r="Q38" s="14">
+        <v>62.001186243563978</v>
+      </c>
+      <c r="Z38" s="9">
         <f t="shared" si="5"/>
-        <v>-2.5971594923925707</v>
-      </c>
-      <c r="R38" s="13">
-        <f>-DEGREES(ATAN((J38-P38)/(K38-Q38)))</f>
-        <v>11.095111708897463</v>
+        <v>-10.862676907493782</v>
+      </c>
+      <c r="AA38" s="9">
+        <f t="shared" si="6"/>
+        <v>202.26818352502269</v>
+      </c>
+      <c r="AB38" s="9">
+        <f t="shared" si="7"/>
+        <v>6.5374490412622421</v>
+      </c>
+      <c r="AC38" s="8">
+        <f t="shared" si="8"/>
+        <v>-3.4376440756897959</v>
       </c>
     </row>
-    <row r="39" spans="3:18" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="H39" s="11">
+    <row r="39" spans="3:29" ht="15.75" x14ac:dyDescent="0.3">
+      <c r="S39" s="6">
         <v>-15</v>
       </c>
-      <c r="I39" s="13">
-        <f>R39-5</f>
-        <v>6.2591524912573213</v>
-      </c>
-      <c r="J39" s="14">
-        <f>$D$5+$D$22*COS(RADIANS(H39))</f>
-        <v>246.80801549544313</v>
-      </c>
-      <c r="K39" s="14">
-        <f>$D$6+$D$22*SIN(RADIANS(H39))</f>
-        <v>60.662910805580267</v>
-      </c>
-      <c r="L39" s="14">
+      <c r="T39" s="8">
+        <f>AC39-H4</f>
+        <v>-3.3455715699963791</v>
+      </c>
+      <c r="U39" s="9">
         <f t="shared" si="0"/>
-        <v>169.60285414048599</v>
-      </c>
-      <c r="M39" s="14">
+        <v>205.81187278706787</v>
+      </c>
+      <c r="V39" s="9">
         <f t="shared" si="1"/>
-        <v>170.59007770195873</v>
-      </c>
-      <c r="N39" s="15">
+        <v>71.647794137080481</v>
+      </c>
+      <c r="W39" s="9">
         <f t="shared" si="2"/>
-        <v>67.074774614900306</v>
-      </c>
-      <c r="O39" s="14">
+        <v>132.52609588558016</v>
+      </c>
+      <c r="X39" s="9">
         <f t="shared" si="3"/>
-        <v>-11.048470734421155</v>
-      </c>
-      <c r="P39" s="14">
+        <v>107.76430822852706</v>
+      </c>
+      <c r="Y39" s="10">
         <f t="shared" si="4"/>
-        <v>259.90558184076343</v>
-      </c>
-      <c r="Q39" s="14">
+        <v>62.344637877102272</v>
+      </c>
+      <c r="Z39" s="9">
         <f t="shared" si="5"/>
-        <v>-5.1280745634650486</v>
-      </c>
-      <c r="R39" s="13">
-        <f>-DEGREES(ATAN((J39-P39)/(K39-Q39)))</f>
-        <v>11.259152491257321</v>
+        <v>-11.734359070917828</v>
+      </c>
+      <c r="AA39" s="9">
+        <f t="shared" si="6"/>
+        <v>201.89709486075594</v>
+      </c>
+      <c r="AB39" s="9">
+        <f t="shared" si="7"/>
+        <v>4.6800816646683501</v>
+      </c>
+      <c r="AC39" s="8">
+        <f t="shared" si="8"/>
+        <v>-3.3455715699963791</v>
       </c>
     </row>
-    <row r="40" spans="3:18" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="C40" s="10" t="s">
+    <row r="40" spans="3:29" ht="15.75" x14ac:dyDescent="0.3">
+      <c r="C40" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D40" s="10"/>
-      <c r="E40" s="10"/>
-      <c r="F40" s="10"/>
-      <c r="H40" s="11">
+      <c r="D40" s="15"/>
+      <c r="E40" s="15"/>
+      <c r="F40" s="15"/>
+      <c r="S40" s="6">
         <v>-16</v>
       </c>
-      <c r="I40" s="13">
-        <f>R40-5</f>
-        <v>6.4327391453079734</v>
-      </c>
-      <c r="J40" s="14">
-        <f>$D$5+$D$22*COS(RADIANS(H40))</f>
-        <v>246.09912905492189</v>
-      </c>
-      <c r="K40" s="14">
-        <f>$D$6+$D$22*SIN(RADIANS(H40))</f>
-        <v>58.106748880120563</v>
-      </c>
-      <c r="L40" s="14">
+      <c r="T40" s="8">
+        <f>AC40-H4</f>
+        <v>-3.249556377075816</v>
+      </c>
+      <c r="U40" s="9">
         <f t="shared" si="0"/>
-        <v>168.46041079557463</v>
-      </c>
-      <c r="M40" s="14">
+        <v>205.30094290621787</v>
+      </c>
+      <c r="V40" s="9">
         <f t="shared" si="1"/>
-        <v>170.60064656723398</v>
-      </c>
-      <c r="N40" s="15">
+        <v>69.805440505590354</v>
+      </c>
+      <c r="W40" s="9">
         <f t="shared" si="2"/>
-        <v>67.047888787356385</v>
-      </c>
-      <c r="O40" s="14">
+        <v>131.47166762094167</v>
+      </c>
+      <c r="X40" s="9">
         <f t="shared" si="3"/>
-        <v>-11.850939177884722</v>
-      </c>
-      <c r="P40" s="14">
+        <v>107.56994225015053</v>
+      </c>
+      <c r="Y40" s="10">
         <f t="shared" si="4"/>
-        <v>259.3959592131452</v>
-      </c>
-      <c r="Q40" s="14">
+        <v>62.679402711730425</v>
+      </c>
+      <c r="Z40" s="9">
         <f t="shared" si="5"/>
-        <v>-7.6442534524930608</v>
-      </c>
-      <c r="R40" s="13">
-        <f>-DEGREES(ATAN((J40-P40)/(K40-Q40)))</f>
-        <v>11.432739145307973</v>
+        <v>-12.604774058967857</v>
+      </c>
+      <c r="AA40" s="9">
+        <f t="shared" si="6"/>
+        <v>201.4983936610127</v>
+      </c>
+      <c r="AB40" s="9">
+        <f t="shared" si="7"/>
+        <v>2.8312617555840944</v>
+      </c>
+      <c r="AC40" s="8">
+        <f t="shared" si="8"/>
+        <v>-3.249556377075816</v>
       </c>
     </row>
-    <row r="41" spans="3:18" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="41" spans="3:29" ht="15.75" x14ac:dyDescent="0.3">
       <c r="C41" s="2" t="s">
         <v>3</v>
       </c>
@@ -4529,57 +4595,57 @@
       <c r="F41" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="H41" s="11">
+      <c r="S41" s="6">
         <v>-17</v>
       </c>
-      <c r="I41" s="13">
-        <f>R41-5</f>
-        <v>6.6161782184459792</v>
-      </c>
-      <c r="J41" s="14">
-        <f>$D$5+$D$22*COS(RADIANS(H41))</f>
-        <v>245.34573940439648</v>
-      </c>
-      <c r="K41" s="14">
-        <f>$D$6+$D$22*SIN(RADIANS(H41))</f>
-        <v>55.563348044780994</v>
-      </c>
-      <c r="L41" s="14">
+      <c r="T41" s="8">
+        <f>AC41-H4</f>
+        <v>-3.1495122601440277</v>
+      </c>
+      <c r="U41" s="9">
         <f t="shared" si="0"/>
-        <v>167.31018588969772</v>
-      </c>
-      <c r="M41" s="14">
+        <v>204.75793733808553</v>
+      </c>
+      <c r="V41" s="9">
         <f t="shared" si="1"/>
-        <v>170.6193140568399</v>
-      </c>
-      <c r="N41" s="15">
+        <v>67.972284429423468</v>
+      </c>
+      <c r="W41" s="9">
         <f t="shared" si="2"/>
-        <v>67.000370676388258</v>
-      </c>
-      <c r="O41" s="14">
+        <v>130.40873173849482</v>
+      </c>
+      <c r="X41" s="9">
         <f t="shared" si="3"/>
-        <v>-12.650748010740694</v>
-      </c>
-      <c r="P41" s="14">
+        <v>107.37945588568131</v>
+      </c>
+      <c r="Y41" s="10">
         <f t="shared" si="4"/>
-        <v>258.85301050264133</v>
-      </c>
-      <c r="Q41" s="14">
+        <v>63.005177991138332</v>
+      </c>
+      <c r="Z41" s="9">
         <f t="shared" si="5"/>
-        <v>-10.144746034095775</v>
-      </c>
-      <c r="R41" s="13">
-        <f>-DEGREES(ATAN((J41-P41)/(K41-Q41)))</f>
-        <v>11.616178218445979</v>
+        <v>-13.473837343900618</v>
+      </c>
+      <c r="AA41" s="9">
+        <f t="shared" si="6"/>
+        <v>201.07233739264137</v>
+      </c>
+      <c r="AB41" s="9">
+        <f t="shared" si="7"/>
+        <v>0.99156815195936332</v>
+      </c>
+      <c r="AC41" s="8">
+        <f t="shared" si="8"/>
+        <v>-3.1495122601440277</v>
       </c>
     </row>
-    <row r="42" spans="3:18" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="42" spans="3:29" ht="15.75" x14ac:dyDescent="0.3">
       <c r="C42" s="2" t="s">
         <v>72</v>
       </c>
       <c r="D42" s="2">
         <f>DEGREES(ATAN(D26/(D29-D37)))</f>
-        <v>16.82114488332024</v>
+        <v>16.646794696917905</v>
       </c>
       <c r="E42" s="2" t="s">
         <v>1</v>
@@ -4587,57 +4653,57 @@
       <c r="F42" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="H42" s="11">
+      <c r="S42" s="6">
         <v>-18</v>
       </c>
-      <c r="I42" s="13">
-        <f>R42-5</f>
-        <v>6.8098017279472227</v>
-      </c>
-      <c r="J42" s="14">
-        <f>$D$5+$D$22*COS(RADIANS(H42))</f>
-        <v>244.54807603365271</v>
-      </c>
-      <c r="K42" s="14">
-        <f>$D$6+$D$22*SIN(RADIANS(H42))</f>
-        <v>53.033483044094517</v>
-      </c>
-      <c r="L42" s="14">
+      <c r="T42" s="8">
+        <f>AC42-H4</f>
+        <v>-3.0453460898189029</v>
+      </c>
+      <c r="U42" s="9">
         <f t="shared" si="0"/>
-        <v>166.15237183838016</v>
-      </c>
-      <c r="M42" s="14">
+        <v>204.18302148742703</v>
+      </c>
+      <c r="V42" s="9">
         <f t="shared" si="1"/>
-        <v>170.64640739128006</v>
-      </c>
-      <c r="N42" s="15">
+        <v>66.148884305678848</v>
+      </c>
+      <c r="W42" s="9">
         <f t="shared" si="2"/>
-        <v>66.931335295579359</v>
-      </c>
-      <c r="O42" s="14">
+        <v>129.33740627634418</v>
+      </c>
+      <c r="X42" s="9">
         <f t="shared" si="3"/>
-        <v>-13.447720222275482</v>
-      </c>
-      <c r="P42" s="14">
+        <v>107.19313716191166</v>
+      </c>
+      <c r="Y42" s="10">
         <f t="shared" si="4"/>
-        <v>258.2773213960046</v>
-      </c>
-      <c r="Q42" s="14">
+        <v>63.321649894704983</v>
+      </c>
+      <c r="Z42" s="9">
         <f t="shared" si="5"/>
-        <v>-12.628589888309421</v>
-      </c>
-      <c r="R42" s="13">
-        <f>-DEGREES(ATAN((J42-P42)/(K42-Q42)))</f>
-        <v>11.809801727947223</v>
+        <v>-14.341461429265133</v>
+      </c>
+      <c r="AA42" s="9">
+        <f t="shared" si="6"/>
+        <v>200.61920136420832</v>
+      </c>
+      <c r="AB42" s="9">
+        <f t="shared" si="7"/>
+        <v>-0.83842185100537847</v>
+      </c>
+      <c r="AC42" s="8">
+        <f t="shared" si="8"/>
+        <v>-3.0453460898189029</v>
       </c>
     </row>
-    <row r="43" spans="3:18" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="43" spans="3:29" ht="15.75" x14ac:dyDescent="0.3">
       <c r="C43" s="2" t="s">
         <v>74</v>
       </c>
       <c r="D43" s="2">
         <f>-DEGREES(ATAN((D28 - D36)/(D29-D37)))</f>
-        <v>9.5366656729775681</v>
+        <v>-4.346821528722181</v>
       </c>
       <c r="E43" s="2" t="s">
         <v>1</v>
@@ -4645,57 +4711,57 @@
       <c r="F43" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="H43" s="11">
+      <c r="S43" s="6">
         <v>-19</v>
       </c>
-      <c r="I43" s="13">
-        <f>R43-5</f>
-        <v>7.0139693260434051</v>
-      </c>
-      <c r="J43" s="14">
-        <f>$D$5+$D$22*COS(RADIANS(H43))</f>
-        <v>243.70638191868042</v>
-      </c>
-      <c r="K43" s="14">
-        <f>$D$6+$D$22*SIN(RADIANS(H43))</f>
-        <v>50.517924499447659</v>
-      </c>
-      <c r="L43" s="14">
+      <c r="T43" s="8">
+        <f>AC43-H4</f>
+        <v>-2.9369574917140335</v>
+      </c>
+      <c r="U43" s="9">
         <f t="shared" si="0"/>
-        <v>164.98716527860552</v>
-      </c>
-      <c r="M43" s="14">
+        <v>203.5763704791799</v>
+      </c>
+      <c r="V43" s="9">
         <f t="shared" si="1"/>
-        <v>170.6822606824108</v>
-      </c>
-      <c r="N43" s="15">
+        <v>64.335795559697829</v>
+      </c>
+      <c r="W43" s="9">
         <f t="shared" si="2"/>
-        <v>66.839852545779578</v>
-      </c>
-      <c r="O43" s="14">
+        <v>128.25781144836711</v>
+      </c>
+      <c r="X43" s="9">
         <f t="shared" si="3"/>
-        <v>-14.241668439855225</v>
-      </c>
-      <c r="P43" s="14">
+        <v>107.01128409857317</v>
+      </c>
+      <c r="Y43" s="10">
         <f t="shared" si="4"/>
-        <v>257.66951964176928</v>
-      </c>
-      <c r="Q43" s="14">
+        <v>63.628492639496507</v>
+      </c>
+      <c r="Z43" s="9">
         <f t="shared" si="5"/>
-        <v>-15.094808905936794</v>
-      </c>
-      <c r="R43" s="13">
-        <f>-DEGREES(ATAN((J43-P43)/(K43-Q43)))</f>
-        <v>12.013969326043405</v>
+        <v>-15.207555592343695</v>
+      </c>
+      <c r="AA43" s="9">
+        <f t="shared" si="6"/>
+        <v>200.13927908369681</v>
+      </c>
+      <c r="AB43" s="9">
+        <f t="shared" si="7"/>
+        <v>-2.6581325438183896</v>
+      </c>
+      <c r="AC43" s="8">
+        <f t="shared" si="8"/>
+        <v>-2.9369574917140335</v>
       </c>
     </row>
-    <row r="44" spans="3:18" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="44" spans="3:29" ht="15.75" x14ac:dyDescent="0.3">
       <c r="C44" s="2" t="s">
         <v>77</v>
       </c>
       <c r="D44" s="1">
         <f>(D28-D5)*(D37-D8)-(D29-D6)*(D36-D7)</f>
-        <v>-245.65128126423224</v>
+        <v>340.78423741989997</v>
       </c>
       <c r="E44" s="2" t="s">
         <v>21</v>
@@ -4703,57 +4769,57 @@
       <c r="F44" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="H44" s="11">
+      <c r="S44" s="6">
         <v>-20</v>
       </c>
-      <c r="I44" s="13">
-        <f>R44-5</f>
-        <v>7.2290707264922318</v>
-      </c>
-      <c r="J44" s="14">
-        <f>$D$5+$D$22*COS(RADIANS(H44))</f>
-        <v>242.82091344766073</v>
-      </c>
-      <c r="K44" s="14">
-        <f>$D$6+$D$22*SIN(RADIANS(H44))</f>
-        <v>48.017438674341918</v>
-      </c>
-      <c r="L44" s="14">
+      <c r="T44" s="8">
+        <f>AC44-H4</f>
+        <v>-2.8242384589742762</v>
+      </c>
+      <c r="U44" s="9">
         <f t="shared" si="0"/>
-        <v>163.81476719854746</v>
-      </c>
-      <c r="M44" s="14">
+        <v>202.93816910511799</v>
+      </c>
+      <c r="V44" s="9">
         <f t="shared" si="1"/>
-        <v>170.72721497848661</v>
-      </c>
-      <c r="N44" s="15">
+        <v>62.533570475876253</v>
+      </c>
+      <c r="W44" s="9">
         <f t="shared" si="2"/>
-        <v>66.724943354712622</v>
-      </c>
-      <c r="O44" s="14">
+        <v>127.17006971307123</v>
+      </c>
+      <c r="X44" s="9">
         <f t="shared" si="3"/>
-        <v>-15.032393915621965</v>
-      </c>
-      <c r="P44" s="14">
+        <v>106.83420514015212</v>
+      </c>
+      <c r="Y44" s="10">
         <f t="shared" si="4"/>
-        <v>257.03027733126095</v>
-      </c>
-      <c r="Q44" s="14">
+        <v>63.925367516126919</v>
+      </c>
+      <c r="Z44" s="9">
         <f t="shared" si="5"/>
-        <v>-17.542411676489643</v>
-      </c>
-      <c r="R44" s="13">
-        <f>-DEGREES(ATAN((J44-P44)/(K44-Q44)))</f>
-        <v>12.229070726492232</v>
+        <v>-16.072025608199755</v>
+      </c>
+      <c r="AA44" s="9">
+        <f t="shared" si="6"/>
+        <v>199.63288265343573</v>
+      </c>
+      <c r="AB44" s="9">
+        <f t="shared" si="7"/>
+        <v>-4.4669898312758534</v>
+      </c>
+      <c r="AC44" s="8">
+        <f t="shared" si="8"/>
+        <v>-2.8242384589742762</v>
       </c>
     </row>
-    <row r="45" spans="3:18" x14ac:dyDescent="0.25">
+    <row r="45" spans="3:29" x14ac:dyDescent="0.25">
       <c r="C45" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D45" s="1">
         <f>D5 + (((D7-D5)*(D37-D8)-(D8-D6)*(D36-D7))/D44)*(D28-D5)</f>
-        <v>-7242.6055522764491</v>
+        <v>2880.5245847431356</v>
       </c>
       <c r="E45" s="2" t="s">
         <v>21</v>
@@ -4762,13 +4828,13 @@
         <v>80</v>
       </c>
     </row>
-    <row r="46" spans="3:18" x14ac:dyDescent="0.25">
+    <row r="46" spans="3:29" x14ac:dyDescent="0.25">
       <c r="C46" s="2" t="s">
         <v>78</v>
       </c>
       <c r="D46" s="1">
         <f>D6 + (((D7-D5)*(D37-D8)-(D8-D6)*(D36-D7))/D44)*(D29-D6)</f>
-        <v>-1194.6994675661169</v>
+        <v>100</v>
       </c>
       <c r="E46" s="2" t="s">
         <v>21</v>
@@ -4778,10 +4844,12 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="5">
     <mergeCell ref="C3:F3"/>
     <mergeCell ref="C18:F18"/>
     <mergeCell ref="C40:F40"/>
+    <mergeCell ref="H3:P3"/>
+    <mergeCell ref="H4:P4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>